<commit_message>
Add database test cases and constraint testing results
</commit_message>
<xml_diff>
--- a/Testcase_KTPM.xlsx
+++ b/Testcase_KTPM.xlsx
@@ -4,10 +4,10 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Cover" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="Database" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="Borrow" sheetId="3" r:id="rId6"/>
-    <sheet state="visible" name="Return" sheetId="4" r:id="rId7"/>
-    <sheet state="visible" name="Search" sheetId="5" r:id="rId8"/>
+    <sheet state="visible" name="Cơ sở dữ liệu" sheetId="2" r:id="rId5"/>
+    <sheet state="visible" name="Mượn sách" sheetId="3" r:id="rId6"/>
+    <sheet state="visible" name="Trả sách" sheetId="4" r:id="rId7"/>
+    <sheet state="visible" name="Tìm kiếm sách" sheetId="5" r:id="rId8"/>
     <sheet state="visible" name="Test Report" sheetId="6" r:id="rId9"/>
   </sheets>
   <externalReferences>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="76">
   <si>
     <t>TEST CASE</t>
   </si>
@@ -93,6 +93,160 @@
     <t>Thái Hùng</t>
   </si>
   <si>
+    <t>1.1</t>
+  </si>
+  <si>
+    <t>Database sheet</t>
+  </si>
+  <si>
+    <t>Add database test cases</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Tahoma"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="10.0"/>
+      </rPr>
+      <t>System Name</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="ＭＳ Ｐゴシック"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="10.0"/>
+      </rPr>
+      <t>：</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Tahoma"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="10.0"/>
+      </rPr>
+      <t>Module Code</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="MS Gothic"/>
+        <b/>
+        <color theme="1"/>
+        <sz val="10.0"/>
+      </rPr>
+      <t>：</t>
+    </r>
+  </si>
+  <si>
+    <t>DB01 - Database Testing</t>
+  </si>
+  <si>
+    <t>Test requirement:</t>
+  </si>
+  <si>
+    <t>DBR1 - Kiểm thử cơ sở dữ liệu</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Number of test cases:</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Test Case Description</t>
+  </si>
+  <si>
+    <t>Test Case Procedure</t>
+  </si>
+  <si>
+    <t>Expected Results</t>
+  </si>
+  <si>
+    <t>Actual Results</t>
+  </si>
+  <si>
+    <t>Test date</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Kiểm thử kết nối database</t>
+  </si>
+  <si>
+    <t>TC01</t>
+  </si>
+  <si>
+    <t>Kiểm tra kết nối Database thành công</t>
+  </si>
+  <si>
+    <t>Mở MySQL Workbench và chạy câu lệnh: 
+SELECT 1;
+SELECT * FROM user</t>
+  </si>
+  <si>
+    <t>Kết nối database thành công và các câu lệnh SELECT thực thi không lỗi</t>
+  </si>
+  <si>
+    <t>Kiểm thử ràng buộc dữ liệu</t>
+  </si>
+  <si>
+    <t>TC02</t>
+  </si>
+  <si>
+    <t>Kiểm tra ràng buộc NOT NULL của cột username trong bảng user</t>
+  </si>
+  <si>
+    <t>Mở MySQL Workbench và chạy câu lệnh: 
+INSERT INTO user(username) VALUES(NULL);</t>
+  </si>
+  <si>
+    <t>Database từ chối insert dữ liệu NULL vào cột username</t>
+  </si>
+  <si>
+    <t>TC03</t>
+  </si>
+  <si>
+    <t>Kiểm tra ràng buộc PRIMARY KEY của bảng user</t>
+  </si>
+  <si>
+    <t>Mở MySQL Workbench và chạy câu lệnh: 
+INSERT INTO user(id, name, username, password) VALUES(10, 'Hung','hung01', 'Abc123');
+INSERT INTO user(id, name, username, password) VALUES(10, 'Huy','huy01', 'Abc123');</t>
+  </si>
+  <si>
+    <t>Database từ chối insert record thứ hai do trùng khóa chính</t>
+  </si>
+  <si>
+    <t>TC04</t>
+  </si>
+  <si>
+    <t>Kiểm tra ràng buộc FOREIGN KEY bảng borrow với user</t>
+  </si>
+  <si>
+    <t>Mở MySQL Workbench và chạy câu lệnh: 
+INSERT INTO borrow(user_id) VALUES(999);</t>
+  </si>
+  <si>
+    <t>Database từ chối insert do user_id không tồn tại</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <rFont val="Tahoma"/>
@@ -139,86 +293,7 @@
     <t>CR100 - Export to excel</t>
   </si>
   <si>
-    <t>Test requirement:</t>
-  </si>
-  <si>
     <t xml:space="preserve">CR1 - </t>
-  </si>
-  <si>
-    <t>Pass</t>
-  </si>
-  <si>
-    <t>Pending</t>
-  </si>
-  <si>
-    <t>Fail</t>
-  </si>
-  <si>
-    <t>Number of test cases:</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Test Case Description</t>
-  </si>
-  <si>
-    <t>Test Case Procedure</t>
-  </si>
-  <si>
-    <t>Expected Results</t>
-  </si>
-  <si>
-    <t>Actual Results</t>
-  </si>
-  <si>
-    <t>Test date</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Note</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Tahoma"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="10.0"/>
-      </rPr>
-      <t>System Name</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="ＭＳ Ｐゴシック"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="10.0"/>
-      </rPr>
-      <t>：</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Tahoma"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="10.0"/>
-      </rPr>
-      <t>Module Code</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="MS Gothic"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="10.0"/>
-      </rPr>
-      <t>：</t>
-    </r>
   </si>
   <si>
     <r>
@@ -335,9 +410,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy"/>
-    <numFmt numFmtId="165" formatCode="0.000"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="d.m"/>
+    <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yy"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -969,7 +1045,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="138">
+  <cellXfs count="150">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -977,7 +1053,7 @@
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
@@ -994,7 +1070,7 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="3" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="5" fillId="3" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="6" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1006,7 +1082,7 @@
     <xf borderId="7" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="8" fillId="0" fontId="4" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="4" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -1036,7 +1112,7 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="8" fillId="0" fontId="4" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1045,7 +1121,7 @@
     <xf borderId="9" fillId="0" fontId="4" numFmtId="15" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="8" fillId="0" fontId="4" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf borderId="9" fillId="0" fontId="4" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -1060,7 +1136,7 @@
     <xf borderId="10" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="11" fillId="0" fontId="4" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf borderId="12" fillId="0" fontId="4" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
@@ -1092,6 +1168,9 @@
     <xf borderId="20" fillId="2" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" wrapText="1"/>
     </xf>
+    <xf borderId="2" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -1106,12 +1185,12 @@
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="25" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="26" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="27" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="25" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -1187,31 +1266,64 @@
     <xf borderId="45" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="25" fillId="6" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="top"/>
     </xf>
-    <xf borderId="28" fillId="0" fontId="9" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+    <xf borderId="28" fillId="0" fontId="9" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="28" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="28" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="25" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="45" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="26" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="25" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="28" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="39" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="25" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="25" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="26" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="25" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="25" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="25" fillId="6" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="28" fillId="0" fontId="9" numFmtId="166" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="28" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="25" fillId="6" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -1237,8 +1349,8 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="8" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="8" fillId="0" fontId="4" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="5" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -1319,7 +1431,120 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2895600" cy="1533525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image4.png"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2886075" cy="1533525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image3.png"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2895600" cy="1533525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image2.png"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2895600" cy="1533525"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.png"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1627,7 +1852,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="5">
-        <v>1.0</v>
+        <v>46023.0</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="2"/>
@@ -1947,12 +2172,24 @@
     </row>
     <row r="13" ht="13.5" customHeight="1">
       <c r="A13" s="13"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="22"/>
+      <c r="B13" s="18">
+        <v>46115.0</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="E13" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" s="25" t="s">
+        <v>18</v>
+      </c>
       <c r="H13" s="23"/>
       <c r="I13" s="13"/>
       <c r="J13" s="13"/>
@@ -29705,477 +29942,513 @@
     </row>
     <row r="3" ht="15.0" customHeight="1">
       <c r="A3" s="51" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>20</v>
+      <c r="B3" s="52" t="s">
+        <v>4</v>
       </c>
       <c r="C3" s="9"/>
       <c r="D3" s="10"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="53"/>
-      <c r="J3" s="54"/>
-      <c r="K3" s="55"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="57"/>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="57"/>
-      <c r="W3" s="57"/>
-      <c r="X3" s="57"/>
-      <c r="Y3" s="57"/>
-      <c r="Z3" s="57"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="53"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
+      <c r="L3" s="57"/>
+      <c r="M3" s="58"/>
+      <c r="N3" s="58"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="58"/>
+      <c r="Q3" s="58"/>
+      <c r="R3" s="58"/>
+      <c r="S3" s="58"/>
+      <c r="T3" s="58"/>
+      <c r="U3" s="58"/>
+      <c r="V3" s="58"/>
+      <c r="W3" s="58"/>
+      <c r="X3" s="58"/>
+      <c r="Y3" s="58"/>
+      <c r="Z3" s="58"/>
     </row>
     <row r="4" ht="13.5" customHeight="1">
-      <c r="A4" s="58" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="59" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="60"/>
-      <c r="D4" s="61"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="52"/>
-      <c r="I4" s="53"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="55"/>
-      <c r="L4" s="56"/>
-      <c r="M4" s="57"/>
-      <c r="N4" s="57"/>
-      <c r="O4" s="57"/>
-      <c r="P4" s="57"/>
-      <c r="Q4" s="57"/>
-      <c r="R4" s="57"/>
-      <c r="S4" s="57"/>
-      <c r="T4" s="57"/>
-      <c r="U4" s="57"/>
-      <c r="V4" s="57"/>
-      <c r="W4" s="57"/>
-      <c r="X4" s="57"/>
-      <c r="Y4" s="57"/>
-      <c r="Z4" s="57"/>
-    </row>
-    <row r="5" ht="13.5" customHeight="1">
-      <c r="A5" s="58" t="s">
+      <c r="A4" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="62" t="s">
+      <c r="B4" s="60" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="60"/>
-      <c r="D5" s="61"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
-      <c r="I5" s="64"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="55"/>
-      <c r="L5" s="65"/>
-      <c r="M5" s="66"/>
-      <c r="N5" s="66"/>
-      <c r="O5" s="66"/>
-      <c r="P5" s="66"/>
-      <c r="Q5" s="66"/>
-      <c r="R5" s="66"/>
-      <c r="S5" s="66"/>
-      <c r="T5" s="66"/>
-      <c r="U5" s="66"/>
-      <c r="V5" s="66"/>
-      <c r="W5" s="66"/>
-      <c r="X5" s="66"/>
-      <c r="Y5" s="66"/>
-      <c r="Z5" s="66"/>
-    </row>
-    <row r="6" ht="15.0" customHeight="1">
-      <c r="A6" s="67" t="s">
+      <c r="C4" s="61"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="56"/>
+      <c r="L4" s="57"/>
+      <c r="M4" s="58"/>
+      <c r="N4" s="58"/>
+      <c r="O4" s="58"/>
+      <c r="P4" s="58"/>
+      <c r="Q4" s="58"/>
+      <c r="R4" s="58"/>
+      <c r="S4" s="58"/>
+      <c r="T4" s="58"/>
+      <c r="U4" s="58"/>
+      <c r="V4" s="58"/>
+      <c r="W4" s="58"/>
+      <c r="X4" s="58"/>
+      <c r="Y4" s="58"/>
+      <c r="Z4" s="58"/>
+    </row>
+    <row r="5" ht="13.5" customHeight="1">
+      <c r="A5" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="68">
-        <f>COUNTIF(J12:J17,"Pass")</f>
+      <c r="B5" s="63" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="61"/>
+      <c r="D5" s="62"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="65"/>
+      <c r="J5" s="55"/>
+      <c r="K5" s="56"/>
+      <c r="L5" s="66"/>
+      <c r="M5" s="67"/>
+      <c r="N5" s="67"/>
+      <c r="O5" s="67"/>
+      <c r="P5" s="67"/>
+      <c r="Q5" s="67"/>
+      <c r="R5" s="67"/>
+      <c r="S5" s="67"/>
+      <c r="T5" s="67"/>
+      <c r="U5" s="67"/>
+      <c r="V5" s="67"/>
+      <c r="W5" s="67"/>
+      <c r="X5" s="67"/>
+      <c r="Y5" s="67"/>
+      <c r="Z5" s="67"/>
+    </row>
+    <row r="6" ht="15.0" customHeight="1">
+      <c r="A6" s="68" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="69">
+        <f>COUNTIF(J12:J16,"Pass")</f>
         <v>3</v>
       </c>
-      <c r="C6" s="69" t="s">
-        <v>26</v>
+      <c r="C6" s="70" t="s">
+        <v>28</v>
       </c>
-      <c r="D6" s="70">
+      <c r="D6" s="71">
         <f>COUNTIF(J10:J736,"Pending")</f>
         <v>0</v>
       </c>
-      <c r="E6" s="71"/>
-      <c r="F6" s="71"/>
-      <c r="G6" s="71"/>
-      <c r="H6" s="71"/>
-      <c r="I6" s="53"/>
-      <c r="J6" s="54"/>
-      <c r="K6" s="55"/>
-      <c r="L6" s="56"/>
-      <c r="M6" s="57"/>
-      <c r="N6" s="57"/>
-      <c r="O6" s="57"/>
-      <c r="P6" s="57"/>
-      <c r="Q6" s="57"/>
-      <c r="R6" s="57"/>
-      <c r="S6" s="57"/>
-      <c r="T6" s="57"/>
-      <c r="U6" s="57"/>
-      <c r="V6" s="57"/>
-      <c r="W6" s="57"/>
-      <c r="X6" s="57"/>
-      <c r="Y6" s="57"/>
-      <c r="Z6" s="57"/>
+      <c r="E6" s="72"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="72"/>
+      <c r="H6" s="72"/>
+      <c r="I6" s="54"/>
+      <c r="J6" s="55"/>
+      <c r="K6" s="56"/>
+      <c r="L6" s="57"/>
+      <c r="M6" s="58"/>
+      <c r="N6" s="58"/>
+      <c r="O6" s="58"/>
+      <c r="P6" s="58"/>
+      <c r="Q6" s="58"/>
+      <c r="R6" s="58"/>
+      <c r="S6" s="58"/>
+      <c r="T6" s="58"/>
+      <c r="U6" s="58"/>
+      <c r="V6" s="58"/>
+      <c r="W6" s="58"/>
+      <c r="X6" s="58"/>
+      <c r="Y6" s="58"/>
+      <c r="Z6" s="58"/>
     </row>
     <row r="7" ht="15.0" customHeight="1">
-      <c r="A7" s="72" t="s">
-        <v>27</v>
+      <c r="A7" s="73" t="s">
+        <v>29</v>
       </c>
-      <c r="B7" s="73">
-        <f>COUNTIF(J12:J17,"Fail")</f>
+      <c r="B7" s="74">
+        <f>COUNTIF(J12:J16,"Fail")</f>
         <v>0</v>
       </c>
-      <c r="C7" s="74" t="s">
-        <v>28</v>
+      <c r="C7" s="75" t="s">
+        <v>30</v>
       </c>
-      <c r="D7" s="75">
-        <f>COUNTA(A12:A17) -15</f>
-        <v>-15</v>
+      <c r="D7" s="76">
+        <f>COUNTA(A12:A16) -15</f>
+        <v>-10</v>
       </c>
-      <c r="E7" s="76"/>
-      <c r="F7" s="76"/>
-      <c r="G7" s="76"/>
-      <c r="H7" s="76"/>
-      <c r="I7" s="53"/>
-      <c r="J7" s="54"/>
-      <c r="K7" s="55"/>
-      <c r="L7" s="56"/>
-      <c r="M7" s="57"/>
-      <c r="N7" s="57"/>
-      <c r="O7" s="57"/>
-      <c r="P7" s="57"/>
-      <c r="Q7" s="57"/>
-      <c r="R7" s="57"/>
-      <c r="S7" s="57"/>
-      <c r="T7" s="57"/>
-      <c r="U7" s="57"/>
-      <c r="V7" s="57"/>
-      <c r="W7" s="57"/>
-      <c r="X7" s="57"/>
-      <c r="Y7" s="57"/>
-      <c r="Z7" s="57"/>
+      <c r="E7" s="77"/>
+      <c r="F7" s="77"/>
+      <c r="G7" s="77"/>
+      <c r="H7" s="77"/>
+      <c r="I7" s="54"/>
+      <c r="J7" s="55"/>
+      <c r="K7" s="56"/>
+      <c r="L7" s="57"/>
+      <c r="M7" s="58"/>
+      <c r="N7" s="58"/>
+      <c r="O7" s="58"/>
+      <c r="P7" s="58"/>
+      <c r="Q7" s="58"/>
+      <c r="R7" s="58"/>
+      <c r="S7" s="58"/>
+      <c r="T7" s="58"/>
+      <c r="U7" s="58"/>
+      <c r="V7" s="58"/>
+      <c r="W7" s="58"/>
+      <c r="X7" s="58"/>
+      <c r="Y7" s="58"/>
+      <c r="Z7" s="58"/>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="77"/>
+      <c r="A8" s="78"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
-      <c r="D8" s="78"/>
-      <c r="E8" s="71"/>
-      <c r="F8" s="71"/>
-      <c r="G8" s="71"/>
-      <c r="H8" s="71"/>
-      <c r="I8" s="71"/>
-      <c r="J8" s="79"/>
-      <c r="K8" s="79"/>
-      <c r="L8" s="56"/>
-      <c r="M8" s="57"/>
-      <c r="N8" s="57"/>
-      <c r="O8" s="57"/>
-      <c r="P8" s="57"/>
-      <c r="Q8" s="57"/>
-      <c r="R8" s="57"/>
-      <c r="S8" s="57"/>
-      <c r="T8" s="57"/>
-      <c r="U8" s="57"/>
-      <c r="V8" s="57"/>
-      <c r="W8" s="57"/>
-      <c r="X8" s="57"/>
-      <c r="Y8" s="57"/>
-      <c r="Z8" s="57"/>
+      <c r="D8" s="79"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="72"/>
+      <c r="H8" s="72"/>
+      <c r="I8" s="72"/>
+      <c r="J8" s="80"/>
+      <c r="K8" s="80"/>
+      <c r="L8" s="57"/>
+      <c r="M8" s="58"/>
+      <c r="N8" s="58"/>
+      <c r="O8" s="58"/>
+      <c r="P8" s="58"/>
+      <c r="Q8" s="58"/>
+      <c r="R8" s="58"/>
+      <c r="S8" s="58"/>
+      <c r="T8" s="58"/>
+      <c r="U8" s="58"/>
+      <c r="V8" s="58"/>
+      <c r="W8" s="58"/>
+      <c r="X8" s="58"/>
+      <c r="Y8" s="58"/>
+      <c r="Z8" s="58"/>
     </row>
     <row r="9" ht="12.0" customHeight="1">
-      <c r="A9" s="80" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="81" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="80" t="s">
+      <c r="A9" s="81" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="82" t="s">
+      <c r="B9" s="82" t="s">
         <v>32</v>
+      </c>
+      <c r="C9" s="81" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="83" t="s">
+        <v>34</v>
       </c>
       <c r="E9" s="42"/>
       <c r="F9" s="42"/>
-      <c r="G9" s="83"/>
-      <c r="H9" s="80" t="s">
-        <v>33</v>
-      </c>
-      <c r="I9" s="84" t="s">
-        <v>34</v>
-      </c>
-      <c r="J9" s="84" t="s">
+      <c r="G9" s="84"/>
+      <c r="H9" s="81" t="s">
         <v>35</v>
       </c>
-      <c r="K9" s="84" t="s">
+      <c r="I9" s="85" t="s">
         <v>36</v>
       </c>
-      <c r="L9" s="85"/>
-      <c r="M9" s="86"/>
-      <c r="N9" s="86"/>
-      <c r="O9" s="86"/>
-      <c r="P9" s="86"/>
-      <c r="Q9" s="86"/>
-      <c r="R9" s="86"/>
-      <c r="S9" s="86"/>
-      <c r="T9" s="86"/>
-      <c r="U9" s="86"/>
-      <c r="V9" s="86"/>
-      <c r="W9" s="86"/>
-      <c r="X9" s="86"/>
-      <c r="Y9" s="86"/>
-      <c r="Z9" s="86"/>
+      <c r="J9" s="85" t="s">
+        <v>37</v>
+      </c>
+      <c r="K9" s="85" t="s">
+        <v>38</v>
+      </c>
+      <c r="L9" s="86"/>
+      <c r="M9" s="87"/>
+      <c r="N9" s="87"/>
+      <c r="O9" s="87"/>
+      <c r="P9" s="87"/>
+      <c r="Q9" s="87"/>
+      <c r="R9" s="87"/>
+      <c r="S9" s="87"/>
+      <c r="T9" s="87"/>
+      <c r="U9" s="87"/>
+      <c r="V9" s="87"/>
+      <c r="W9" s="87"/>
+      <c r="X9" s="87"/>
+      <c r="Y9" s="87"/>
+      <c r="Z9" s="87"/>
     </row>
     <row r="10" ht="12.0" customHeight="1">
-      <c r="A10" s="87"/>
-      <c r="B10" s="87"/>
-      <c r="C10" s="87"/>
-      <c r="D10" s="88"/>
-      <c r="E10" s="89"/>
-      <c r="F10" s="89"/>
-      <c r="G10" s="90"/>
-      <c r="H10" s="87"/>
-      <c r="I10" s="87"/>
-      <c r="J10" s="87"/>
-      <c r="K10" s="87"/>
-      <c r="L10" s="56"/>
-      <c r="M10" s="57"/>
-      <c r="N10" s="57"/>
-      <c r="O10" s="57"/>
-      <c r="P10" s="57"/>
-      <c r="Q10" s="57"/>
-      <c r="R10" s="57"/>
-      <c r="S10" s="57"/>
-      <c r="T10" s="57"/>
-      <c r="U10" s="57"/>
-      <c r="V10" s="57"/>
-      <c r="W10" s="57"/>
-      <c r="X10" s="57"/>
-      <c r="Y10" s="57"/>
-      <c r="Z10" s="57"/>
+      <c r="A10" s="88"/>
+      <c r="B10" s="88"/>
+      <c r="C10" s="88"/>
+      <c r="D10" s="89"/>
+      <c r="E10" s="90"/>
+      <c r="F10" s="90"/>
+      <c r="G10" s="91"/>
+      <c r="H10" s="88"/>
+      <c r="I10" s="88"/>
+      <c r="J10" s="88"/>
+      <c r="K10" s="88"/>
+      <c r="L10" s="57"/>
+      <c r="M10" s="58"/>
+      <c r="N10" s="58"/>
+      <c r="O10" s="58"/>
+      <c r="P10" s="58"/>
+      <c r="Q10" s="58"/>
+      <c r="R10" s="58"/>
+      <c r="S10" s="58"/>
+      <c r="T10" s="58"/>
+      <c r="U10" s="58"/>
+      <c r="V10" s="58"/>
+      <c r="W10" s="58"/>
+      <c r="X10" s="58"/>
+      <c r="Y10" s="58"/>
+      <c r="Z10" s="58"/>
     </row>
     <row r="11" ht="13.5" customHeight="1">
-      <c r="A11" s="91"/>
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
-      <c r="I11" s="60"/>
-      <c r="J11" s="60"/>
-      <c r="K11" s="92"/>
-      <c r="L11" s="93"/>
-      <c r="M11" s="93"/>
-      <c r="N11" s="93"/>
-      <c r="O11" s="93"/>
-      <c r="P11" s="93"/>
-      <c r="Q11" s="93"/>
-      <c r="R11" s="93"/>
-      <c r="S11" s="93"/>
-      <c r="T11" s="93"/>
-      <c r="U11" s="93"/>
-      <c r="V11" s="93"/>
-      <c r="W11" s="93"/>
-      <c r="X11" s="93"/>
-      <c r="Y11" s="93"/>
-      <c r="Z11" s="93"/>
+      <c r="A11" s="92"/>
+      <c r="B11" s="61"/>
+      <c r="C11" s="61"/>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
+      <c r="I11" s="61"/>
+      <c r="J11" s="61"/>
+      <c r="K11" s="93"/>
+      <c r="L11" s="94"/>
+      <c r="M11" s="94"/>
+      <c r="N11" s="94"/>
+      <c r="O11" s="94"/>
+      <c r="P11" s="94"/>
+      <c r="Q11" s="94"/>
+      <c r="R11" s="94"/>
+      <c r="S11" s="94"/>
+      <c r="T11" s="94"/>
+      <c r="U11" s="94"/>
+      <c r="V11" s="94"/>
+      <c r="W11" s="94"/>
+      <c r="X11" s="94"/>
+      <c r="Y11" s="94"/>
+      <c r="Z11" s="94"/>
     </row>
     <row r="12" ht="13.5" customHeight="1">
-      <c r="A12" s="94"/>
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="60"/>
-      <c r="I12" s="60"/>
-      <c r="J12" s="60"/>
-      <c r="K12" s="92"/>
-      <c r="L12" s="95"/>
-      <c r="M12" s="95"/>
-      <c r="N12" s="95"/>
-      <c r="O12" s="95"/>
-      <c r="P12" s="95"/>
-      <c r="Q12" s="95"/>
-      <c r="R12" s="95"/>
-      <c r="S12" s="95"/>
-      <c r="T12" s="95"/>
-      <c r="U12" s="95"/>
-      <c r="V12" s="95"/>
-      <c r="W12" s="95"/>
-      <c r="X12" s="95"/>
-      <c r="Y12" s="95"/>
-      <c r="Z12" s="95"/>
-    </row>
-    <row r="13" ht="13.5" customHeight="1" outlineLevel="1">
-      <c r="A13" s="96"/>
-      <c r="B13" s="97"/>
-      <c r="C13" s="98"/>
-      <c r="D13" s="99"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="100"/>
-      <c r="H13" s="101"/>
-      <c r="I13" s="102"/>
-      <c r="J13" s="98" t="s">
-        <v>25</v>
+      <c r="A12" s="95" t="s">
+        <v>39</v>
       </c>
-      <c r="K13" s="98"/>
-      <c r="L13" s="95"/>
-      <c r="M13" s="95"/>
-      <c r="N13" s="95"/>
-      <c r="O13" s="95"/>
-      <c r="P13" s="95"/>
-      <c r="Q13" s="95"/>
-      <c r="R13" s="95"/>
-      <c r="S13" s="95"/>
-      <c r="T13" s="95"/>
-      <c r="U13" s="95"/>
-      <c r="V13" s="95"/>
-      <c r="W13" s="95"/>
-      <c r="X13" s="95"/>
-      <c r="Y13" s="95"/>
-      <c r="Z13" s="95"/>
-    </row>
-    <row r="14" ht="13.5" customHeight="1" outlineLevel="1">
-      <c r="A14" s="103"/>
-      <c r="B14" s="60"/>
-      <c r="C14" s="104"/>
-      <c r="D14" s="105"/>
-      <c r="E14" s="105"/>
-      <c r="F14" s="105"/>
-      <c r="G14" s="105"/>
-      <c r="H14" s="105"/>
-      <c r="I14" s="105"/>
-      <c r="J14" s="105"/>
-      <c r="K14" s="106"/>
-      <c r="L14" s="95"/>
-      <c r="M14" s="95"/>
-      <c r="N14" s="95"/>
-      <c r="O14" s="95"/>
-      <c r="P14" s="95"/>
-      <c r="Q14" s="95"/>
-      <c r="R14" s="95"/>
-      <c r="S14" s="95"/>
-      <c r="T14" s="95"/>
-      <c r="U14" s="95"/>
-      <c r="V14" s="95"/>
-      <c r="W14" s="95"/>
-      <c r="X14" s="95"/>
-      <c r="Y14" s="95"/>
-      <c r="Z14" s="95"/>
-    </row>
-    <row r="15" ht="63.75" customHeight="1" outlineLevel="1">
-      <c r="A15" s="96"/>
-      <c r="B15" s="107"/>
-      <c r="C15" s="108"/>
-      <c r="D15" s="109"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="60"/>
-      <c r="G15" s="100"/>
-      <c r="H15" s="101"/>
-      <c r="I15" s="99"/>
-      <c r="J15" s="98" t="s">
-        <v>25</v>
+      <c r="B12" s="61"/>
+      <c r="C12" s="61"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="61"/>
+      <c r="I12" s="61"/>
+      <c r="J12" s="61"/>
+      <c r="K12" s="93"/>
+      <c r="L12" s="96"/>
+      <c r="M12" s="96"/>
+      <c r="N12" s="96"/>
+      <c r="O12" s="96"/>
+      <c r="P12" s="96"/>
+      <c r="Q12" s="96"/>
+      <c r="R12" s="96"/>
+      <c r="S12" s="96"/>
+      <c r="T12" s="96"/>
+      <c r="U12" s="96"/>
+      <c r="V12" s="96"/>
+      <c r="W12" s="96"/>
+      <c r="X12" s="96"/>
+      <c r="Y12" s="96"/>
+      <c r="Z12" s="96"/>
+    </row>
+    <row r="13" ht="129.0" customHeight="1" outlineLevel="1">
+      <c r="A13" s="97" t="s">
+        <v>40</v>
       </c>
-      <c r="K15" s="98"/>
-      <c r="L15" s="95"/>
-      <c r="M15" s="95"/>
-      <c r="N15" s="95"/>
-      <c r="O15" s="95"/>
-      <c r="P15" s="95"/>
-      <c r="Q15" s="95"/>
-      <c r="R15" s="95"/>
-      <c r="S15" s="95"/>
-      <c r="T15" s="95"/>
-      <c r="U15" s="95"/>
-      <c r="V15" s="95"/>
-      <c r="W15" s="95"/>
-      <c r="X15" s="95"/>
-      <c r="Y15" s="95"/>
-      <c r="Z15" s="95"/>
-    </row>
-    <row r="16" ht="13.5" customHeight="1" outlineLevel="1">
-      <c r="A16" s="103"/>
-      <c r="B16" s="60"/>
-      <c r="C16" s="104"/>
-      <c r="D16" s="105"/>
-      <c r="E16" s="105"/>
-      <c r="F16" s="105"/>
-      <c r="G16" s="105"/>
-      <c r="H16" s="105"/>
-      <c r="I16" s="105"/>
-      <c r="J16" s="105"/>
-      <c r="K16" s="106"/>
-      <c r="L16" s="95"/>
-      <c r="M16" s="95"/>
-      <c r="N16" s="95"/>
-      <c r="O16" s="95"/>
-      <c r="P16" s="95"/>
-      <c r="Q16" s="95"/>
-      <c r="R16" s="95"/>
-      <c r="S16" s="95"/>
-      <c r="T16" s="95"/>
-      <c r="U16" s="95"/>
-      <c r="V16" s="95"/>
-      <c r="W16" s="95"/>
-      <c r="X16" s="95"/>
-      <c r="Y16" s="95"/>
-      <c r="Z16" s="95"/>
-    </row>
-    <row r="17" ht="63.75" customHeight="1" outlineLevel="1">
-      <c r="A17" s="96"/>
-      <c r="B17" s="110"/>
-      <c r="C17" s="98"/>
-      <c r="D17" s="109"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="60"/>
-      <c r="G17" s="100"/>
-      <c r="H17" s="101"/>
-      <c r="I17" s="99"/>
-      <c r="J17" s="98" t="s">
-        <v>25</v>
+      <c r="B13" s="98" t="s">
+        <v>41</v>
       </c>
-      <c r="K17" s="98"/>
-      <c r="L17" s="95"/>
-      <c r="M17" s="95"/>
-      <c r="N17" s="95"/>
-      <c r="O17" s="95"/>
-      <c r="P17" s="95"/>
-      <c r="Q17" s="95"/>
-      <c r="R17" s="95"/>
-      <c r="S17" s="95"/>
-      <c r="T17" s="95"/>
-      <c r="U17" s="95"/>
-      <c r="V17" s="95"/>
-      <c r="W17" s="95"/>
-      <c r="X17" s="95"/>
-      <c r="Y17" s="95"/>
-      <c r="Z17" s="95"/>
+      <c r="C13" s="99" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" s="100" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="61"/>
+      <c r="F13" s="61"/>
+      <c r="G13" s="101"/>
+      <c r="H13" s="102"/>
+      <c r="I13" s="103"/>
+      <c r="J13" s="104" t="s">
+        <v>27</v>
+      </c>
+      <c r="K13" s="104"/>
+      <c r="L13" s="96"/>
+      <c r="M13" s="96"/>
+      <c r="N13" s="96"/>
+      <c r="O13" s="96"/>
+      <c r="P13" s="96"/>
+      <c r="Q13" s="96"/>
+      <c r="R13" s="96"/>
+      <c r="S13" s="96"/>
+      <c r="T13" s="96"/>
+      <c r="U13" s="96"/>
+      <c r="V13" s="96"/>
+      <c r="W13" s="96"/>
+      <c r="X13" s="96"/>
+      <c r="Y13" s="96"/>
+      <c r="Z13" s="96"/>
+    </row>
+    <row r="14" ht="13.5" customHeight="1">
+      <c r="A14" s="95" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="61"/>
+      <c r="C14" s="61"/>
+      <c r="D14" s="61"/>
+      <c r="E14" s="61"/>
+      <c r="F14" s="61"/>
+      <c r="G14" s="61"/>
+      <c r="H14" s="61"/>
+      <c r="I14" s="61"/>
+      <c r="J14" s="61"/>
+      <c r="K14" s="93"/>
+      <c r="L14" s="96"/>
+      <c r="M14" s="96"/>
+      <c r="N14" s="96"/>
+      <c r="O14" s="96"/>
+      <c r="P14" s="96"/>
+      <c r="Q14" s="96"/>
+      <c r="R14" s="96"/>
+      <c r="S14" s="96"/>
+      <c r="T14" s="96"/>
+      <c r="U14" s="96"/>
+      <c r="V14" s="96"/>
+      <c r="W14" s="96"/>
+      <c r="X14" s="96"/>
+      <c r="Y14" s="96"/>
+      <c r="Z14" s="96"/>
+    </row>
+    <row r="15" ht="120.75" customHeight="1" outlineLevel="1">
+      <c r="A15" s="97" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="105" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="99" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="106" t="s">
+        <v>48</v>
+      </c>
+      <c r="E15" s="61"/>
+      <c r="F15" s="61"/>
+      <c r="G15" s="101"/>
+      <c r="H15" s="102"/>
+      <c r="I15" s="107"/>
+      <c r="J15" s="104" t="s">
+        <v>27</v>
+      </c>
+      <c r="K15" s="104"/>
+      <c r="L15" s="96"/>
+      <c r="M15" s="96"/>
+      <c r="N15" s="96"/>
+      <c r="O15" s="96"/>
+      <c r="P15" s="96"/>
+      <c r="Q15" s="96"/>
+      <c r="R15" s="96"/>
+      <c r="S15" s="96"/>
+      <c r="T15" s="96"/>
+      <c r="U15" s="96"/>
+      <c r="V15" s="96"/>
+      <c r="W15" s="96"/>
+      <c r="X15" s="96"/>
+      <c r="Y15" s="96"/>
+      <c r="Z15" s="96"/>
+    </row>
+    <row r="16" ht="124.5" customHeight="1" outlineLevel="1">
+      <c r="A16" s="97" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="99" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="99" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16" s="100" t="s">
+        <v>52</v>
+      </c>
+      <c r="E16" s="61"/>
+      <c r="F16" s="61"/>
+      <c r="G16" s="101"/>
+      <c r="H16" s="108"/>
+      <c r="I16" s="107"/>
+      <c r="J16" s="104" t="s">
+        <v>27</v>
+      </c>
+      <c r="K16" s="104"/>
+      <c r="L16" s="96"/>
+      <c r="M16" s="96"/>
+      <c r="N16" s="96"/>
+      <c r="O16" s="96"/>
+      <c r="P16" s="96"/>
+      <c r="Q16" s="96"/>
+      <c r="R16" s="96"/>
+      <c r="S16" s="96"/>
+      <c r="T16" s="96"/>
+      <c r="U16" s="96"/>
+      <c r="V16" s="96"/>
+      <c r="W16" s="96"/>
+      <c r="X16" s="96"/>
+      <c r="Y16" s="96"/>
+      <c r="Z16" s="96"/>
+    </row>
+    <row r="17" ht="124.5" customHeight="1" outlineLevel="1">
+      <c r="A17" s="97" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="99" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="99" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17" s="100" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" s="61"/>
+      <c r="F17" s="93"/>
+      <c r="G17" s="104"/>
+      <c r="H17" s="104"/>
+      <c r="I17" s="104"/>
+      <c r="J17" s="104"/>
+      <c r="K17" s="109"/>
+      <c r="L17" s="96"/>
+      <c r="M17" s="96"/>
+      <c r="N17" s="96"/>
+      <c r="O17" s="96"/>
+      <c r="P17" s="96"/>
+      <c r="Q17" s="96"/>
+      <c r="R17" s="96"/>
+      <c r="S17" s="96"/>
+      <c r="T17" s="96"/>
+      <c r="U17" s="96"/>
+      <c r="V17" s="96"/>
+      <c r="W17" s="96"/>
+      <c r="X17" s="96"/>
+      <c r="Y17" s="96"/>
+      <c r="Z17" s="96"/>
     </row>
     <row r="18" ht="12.0" customHeight="1">
       <c r="J18" s="11"/>
@@ -33142,9 +33415,9 @@
     <mergeCell ref="A11:K11"/>
     <mergeCell ref="A12:K12"/>
     <mergeCell ref="D13:F13"/>
-    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D16:F16"/>
     <mergeCell ref="D15:F15"/>
-    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A14:K14"/>
     <mergeCell ref="D17:F17"/>
     <mergeCell ref="I6:K6"/>
     <mergeCell ref="I7:K7"/>
@@ -33242,477 +33515,477 @@
     </row>
     <row r="3" ht="15.0" customHeight="1">
       <c r="A3" s="51" t="s">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="C3" s="9"/>
       <c r="D3" s="10"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="53"/>
-      <c r="J3" s="54"/>
-      <c r="K3" s="55"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="57"/>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="57"/>
-      <c r="W3" s="57"/>
-      <c r="X3" s="57"/>
-      <c r="Y3" s="57"/>
-      <c r="Z3" s="57"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="53"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
+      <c r="L3" s="57"/>
+      <c r="M3" s="58"/>
+      <c r="N3" s="58"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="58"/>
+      <c r="Q3" s="58"/>
+      <c r="R3" s="58"/>
+      <c r="S3" s="58"/>
+      <c r="T3" s="58"/>
+      <c r="U3" s="58"/>
+      <c r="V3" s="58"/>
+      <c r="W3" s="58"/>
+      <c r="X3" s="58"/>
+      <c r="Y3" s="58"/>
+      <c r="Z3" s="58"/>
     </row>
     <row r="4" ht="13.5" customHeight="1">
-      <c r="A4" s="58" t="s">
-        <v>38</v>
+      <c r="A4" s="59" t="s">
+        <v>59</v>
       </c>
-      <c r="B4" s="59" t="s">
-        <v>22</v>
+      <c r="B4" s="110" t="s">
+        <v>60</v>
       </c>
-      <c r="C4" s="60"/>
-      <c r="D4" s="61"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="52"/>
-      <c r="I4" s="53"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="55"/>
-      <c r="L4" s="56"/>
-      <c r="M4" s="57"/>
-      <c r="N4" s="57"/>
-      <c r="O4" s="57"/>
-      <c r="P4" s="57"/>
-      <c r="Q4" s="57"/>
-      <c r="R4" s="57"/>
-      <c r="S4" s="57"/>
-      <c r="T4" s="57"/>
-      <c r="U4" s="57"/>
-      <c r="V4" s="57"/>
-      <c r="W4" s="57"/>
-      <c r="X4" s="57"/>
-      <c r="Y4" s="57"/>
-      <c r="Z4" s="57"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="56"/>
+      <c r="L4" s="57"/>
+      <c r="M4" s="58"/>
+      <c r="N4" s="58"/>
+      <c r="O4" s="58"/>
+      <c r="P4" s="58"/>
+      <c r="Q4" s="58"/>
+      <c r="R4" s="58"/>
+      <c r="S4" s="58"/>
+      <c r="T4" s="58"/>
+      <c r="U4" s="58"/>
+      <c r="V4" s="58"/>
+      <c r="W4" s="58"/>
+      <c r="X4" s="58"/>
+      <c r="Y4" s="58"/>
+      <c r="Z4" s="58"/>
     </row>
     <row r="5" ht="13.5" customHeight="1">
-      <c r="A5" s="58" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="62" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="60"/>
-      <c r="D5" s="61"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
-      <c r="I5" s="64"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="55"/>
-      <c r="L5" s="65"/>
-      <c r="M5" s="66"/>
-      <c r="N5" s="66"/>
-      <c r="O5" s="66"/>
-      <c r="P5" s="66"/>
-      <c r="Q5" s="66"/>
-      <c r="R5" s="66"/>
-      <c r="S5" s="66"/>
-      <c r="T5" s="66"/>
-      <c r="U5" s="66"/>
-      <c r="V5" s="66"/>
-      <c r="W5" s="66"/>
-      <c r="X5" s="66"/>
-      <c r="Y5" s="66"/>
-      <c r="Z5" s="66"/>
-    </row>
-    <row r="6" ht="15.0" customHeight="1">
-      <c r="A6" s="67" t="s">
+      <c r="A5" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="68">
+      <c r="B5" s="111" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="61"/>
+      <c r="D5" s="62"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="65"/>
+      <c r="J5" s="55"/>
+      <c r="K5" s="56"/>
+      <c r="L5" s="66"/>
+      <c r="M5" s="67"/>
+      <c r="N5" s="67"/>
+      <c r="O5" s="67"/>
+      <c r="P5" s="67"/>
+      <c r="Q5" s="67"/>
+      <c r="R5" s="67"/>
+      <c r="S5" s="67"/>
+      <c r="T5" s="67"/>
+      <c r="U5" s="67"/>
+      <c r="V5" s="67"/>
+      <c r="W5" s="67"/>
+      <c r="X5" s="67"/>
+      <c r="Y5" s="67"/>
+      <c r="Z5" s="67"/>
+    </row>
+    <row r="6" ht="15.0" customHeight="1">
+      <c r="A6" s="68" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="69">
         <f>COUNTIF(J12:J17,"Pass")</f>
         <v>3</v>
       </c>
-      <c r="C6" s="69" t="s">
-        <v>26</v>
+      <c r="C6" s="70" t="s">
+        <v>28</v>
       </c>
-      <c r="D6" s="70">
+      <c r="D6" s="71">
         <f>COUNTIF(J10:J736,"Pending")</f>
         <v>0</v>
       </c>
-      <c r="E6" s="71"/>
-      <c r="F6" s="71"/>
-      <c r="G6" s="71"/>
-      <c r="H6" s="71"/>
-      <c r="I6" s="53"/>
-      <c r="J6" s="54"/>
-      <c r="K6" s="55"/>
-      <c r="L6" s="56"/>
-      <c r="M6" s="57"/>
-      <c r="N6" s="57"/>
-      <c r="O6" s="57"/>
-      <c r="P6" s="57"/>
-      <c r="Q6" s="57"/>
-      <c r="R6" s="57"/>
-      <c r="S6" s="57"/>
-      <c r="T6" s="57"/>
-      <c r="U6" s="57"/>
-      <c r="V6" s="57"/>
-      <c r="W6" s="57"/>
-      <c r="X6" s="57"/>
-      <c r="Y6" s="57"/>
-      <c r="Z6" s="57"/>
+      <c r="E6" s="72"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="72"/>
+      <c r="H6" s="72"/>
+      <c r="I6" s="54"/>
+      <c r="J6" s="55"/>
+      <c r="K6" s="56"/>
+      <c r="L6" s="57"/>
+      <c r="M6" s="58"/>
+      <c r="N6" s="58"/>
+      <c r="O6" s="58"/>
+      <c r="P6" s="58"/>
+      <c r="Q6" s="58"/>
+      <c r="R6" s="58"/>
+      <c r="S6" s="58"/>
+      <c r="T6" s="58"/>
+      <c r="U6" s="58"/>
+      <c r="V6" s="58"/>
+      <c r="W6" s="58"/>
+      <c r="X6" s="58"/>
+      <c r="Y6" s="58"/>
+      <c r="Z6" s="58"/>
     </row>
     <row r="7" ht="15.0" customHeight="1">
-      <c r="A7" s="72" t="s">
-        <v>27</v>
+      <c r="A7" s="73" t="s">
+        <v>29</v>
       </c>
-      <c r="B7" s="73">
+      <c r="B7" s="74">
         <f>COUNTIF(J12:J17,"Fail")</f>
         <v>0</v>
       </c>
-      <c r="C7" s="74" t="s">
-        <v>28</v>
+      <c r="C7" s="75" t="s">
+        <v>30</v>
       </c>
-      <c r="D7" s="75">
+      <c r="D7" s="76">
         <f>COUNTA(A12:A17) -15</f>
         <v>-15</v>
       </c>
-      <c r="E7" s="76"/>
-      <c r="F7" s="76"/>
-      <c r="G7" s="76"/>
-      <c r="H7" s="76"/>
-      <c r="I7" s="53"/>
-      <c r="J7" s="54"/>
-      <c r="K7" s="55"/>
-      <c r="L7" s="56"/>
-      <c r="M7" s="57"/>
-      <c r="N7" s="57"/>
-      <c r="O7" s="57"/>
-      <c r="P7" s="57"/>
-      <c r="Q7" s="57"/>
-      <c r="R7" s="57"/>
-      <c r="S7" s="57"/>
-      <c r="T7" s="57"/>
-      <c r="U7" s="57"/>
-      <c r="V7" s="57"/>
-      <c r="W7" s="57"/>
-      <c r="X7" s="57"/>
-      <c r="Y7" s="57"/>
-      <c r="Z7" s="57"/>
+      <c r="E7" s="77"/>
+      <c r="F7" s="77"/>
+      <c r="G7" s="77"/>
+      <c r="H7" s="77"/>
+      <c r="I7" s="54"/>
+      <c r="J7" s="55"/>
+      <c r="K7" s="56"/>
+      <c r="L7" s="57"/>
+      <c r="M7" s="58"/>
+      <c r="N7" s="58"/>
+      <c r="O7" s="58"/>
+      <c r="P7" s="58"/>
+      <c r="Q7" s="58"/>
+      <c r="R7" s="58"/>
+      <c r="S7" s="58"/>
+      <c r="T7" s="58"/>
+      <c r="U7" s="58"/>
+      <c r="V7" s="58"/>
+      <c r="W7" s="58"/>
+      <c r="X7" s="58"/>
+      <c r="Y7" s="58"/>
+      <c r="Z7" s="58"/>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="77"/>
+      <c r="A8" s="78"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
-      <c r="D8" s="78"/>
-      <c r="E8" s="71"/>
-      <c r="F8" s="71"/>
-      <c r="G8" s="71"/>
-      <c r="H8" s="71"/>
-      <c r="I8" s="71"/>
-      <c r="J8" s="79"/>
-      <c r="K8" s="79"/>
-      <c r="L8" s="56"/>
-      <c r="M8" s="57"/>
-      <c r="N8" s="57"/>
-      <c r="O8" s="57"/>
-      <c r="P8" s="57"/>
-      <c r="Q8" s="57"/>
-      <c r="R8" s="57"/>
-      <c r="S8" s="57"/>
-      <c r="T8" s="57"/>
-      <c r="U8" s="57"/>
-      <c r="V8" s="57"/>
-      <c r="W8" s="57"/>
-      <c r="X8" s="57"/>
-      <c r="Y8" s="57"/>
-      <c r="Z8" s="57"/>
+      <c r="D8" s="79"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="72"/>
+      <c r="H8" s="72"/>
+      <c r="I8" s="72"/>
+      <c r="J8" s="80"/>
+      <c r="K8" s="80"/>
+      <c r="L8" s="57"/>
+      <c r="M8" s="58"/>
+      <c r="N8" s="58"/>
+      <c r="O8" s="58"/>
+      <c r="P8" s="58"/>
+      <c r="Q8" s="58"/>
+      <c r="R8" s="58"/>
+      <c r="S8" s="58"/>
+      <c r="T8" s="58"/>
+      <c r="U8" s="58"/>
+      <c r="V8" s="58"/>
+      <c r="W8" s="58"/>
+      <c r="X8" s="58"/>
+      <c r="Y8" s="58"/>
+      <c r="Z8" s="58"/>
     </row>
     <row r="9" ht="12.0" customHeight="1">
-      <c r="A9" s="80" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="81" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="80" t="s">
+      <c r="A9" s="81" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="82" t="s">
+      <c r="B9" s="82" t="s">
         <v>32</v>
+      </c>
+      <c r="C9" s="81" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="83" t="s">
+        <v>34</v>
       </c>
       <c r="E9" s="42"/>
       <c r="F9" s="42"/>
-      <c r="G9" s="83"/>
-      <c r="H9" s="80" t="s">
-        <v>33</v>
-      </c>
-      <c r="I9" s="84" t="s">
-        <v>34</v>
-      </c>
-      <c r="J9" s="84" t="s">
+      <c r="G9" s="84"/>
+      <c r="H9" s="81" t="s">
         <v>35</v>
       </c>
-      <c r="K9" s="84" t="s">
+      <c r="I9" s="85" t="s">
         <v>36</v>
       </c>
-      <c r="L9" s="85"/>
-      <c r="M9" s="86"/>
-      <c r="N9" s="86"/>
-      <c r="O9" s="86"/>
-      <c r="P9" s="86"/>
-      <c r="Q9" s="86"/>
-      <c r="R9" s="86"/>
-      <c r="S9" s="86"/>
-      <c r="T9" s="86"/>
-      <c r="U9" s="86"/>
-      <c r="V9" s="86"/>
-      <c r="W9" s="86"/>
-      <c r="X9" s="86"/>
-      <c r="Y9" s="86"/>
-      <c r="Z9" s="86"/>
+      <c r="J9" s="85" t="s">
+        <v>37</v>
+      </c>
+      <c r="K9" s="85" t="s">
+        <v>38</v>
+      </c>
+      <c r="L9" s="86"/>
+      <c r="M9" s="87"/>
+      <c r="N9" s="87"/>
+      <c r="O9" s="87"/>
+      <c r="P9" s="87"/>
+      <c r="Q9" s="87"/>
+      <c r="R9" s="87"/>
+      <c r="S9" s="87"/>
+      <c r="T9" s="87"/>
+      <c r="U9" s="87"/>
+      <c r="V9" s="87"/>
+      <c r="W9" s="87"/>
+      <c r="X9" s="87"/>
+      <c r="Y9" s="87"/>
+      <c r="Z9" s="87"/>
     </row>
     <row r="10" ht="12.0" customHeight="1">
-      <c r="A10" s="87"/>
-      <c r="B10" s="87"/>
-      <c r="C10" s="87"/>
-      <c r="D10" s="88"/>
-      <c r="E10" s="89"/>
-      <c r="F10" s="89"/>
-      <c r="G10" s="90"/>
-      <c r="H10" s="87"/>
-      <c r="I10" s="87"/>
-      <c r="J10" s="87"/>
-      <c r="K10" s="87"/>
-      <c r="L10" s="56"/>
-      <c r="M10" s="57"/>
-      <c r="N10" s="57"/>
-      <c r="O10" s="57"/>
-      <c r="P10" s="57"/>
-      <c r="Q10" s="57"/>
-      <c r="R10" s="57"/>
-      <c r="S10" s="57"/>
-      <c r="T10" s="57"/>
-      <c r="U10" s="57"/>
-      <c r="V10" s="57"/>
-      <c r="W10" s="57"/>
-      <c r="X10" s="57"/>
-      <c r="Y10" s="57"/>
-      <c r="Z10" s="57"/>
+      <c r="A10" s="88"/>
+      <c r="B10" s="88"/>
+      <c r="C10" s="88"/>
+      <c r="D10" s="89"/>
+      <c r="E10" s="90"/>
+      <c r="F10" s="90"/>
+      <c r="G10" s="91"/>
+      <c r="H10" s="88"/>
+      <c r="I10" s="88"/>
+      <c r="J10" s="88"/>
+      <c r="K10" s="88"/>
+      <c r="L10" s="57"/>
+      <c r="M10" s="58"/>
+      <c r="N10" s="58"/>
+      <c r="O10" s="58"/>
+      <c r="P10" s="58"/>
+      <c r="Q10" s="58"/>
+      <c r="R10" s="58"/>
+      <c r="S10" s="58"/>
+      <c r="T10" s="58"/>
+      <c r="U10" s="58"/>
+      <c r="V10" s="58"/>
+      <c r="W10" s="58"/>
+      <c r="X10" s="58"/>
+      <c r="Y10" s="58"/>
+      <c r="Z10" s="58"/>
     </row>
     <row r="11" ht="13.5" customHeight="1">
-      <c r="A11" s="91"/>
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
-      <c r="I11" s="60"/>
-      <c r="J11" s="60"/>
-      <c r="K11" s="92"/>
-      <c r="L11" s="93"/>
-      <c r="M11" s="93"/>
-      <c r="N11" s="93"/>
-      <c r="O11" s="93"/>
-      <c r="P11" s="93"/>
-      <c r="Q11" s="93"/>
-      <c r="R11" s="93"/>
-      <c r="S11" s="93"/>
-      <c r="T11" s="93"/>
-      <c r="U11" s="93"/>
-      <c r="V11" s="93"/>
-      <c r="W11" s="93"/>
-      <c r="X11" s="93"/>
-      <c r="Y11" s="93"/>
-      <c r="Z11" s="93"/>
+      <c r="A11" s="92"/>
+      <c r="B11" s="61"/>
+      <c r="C11" s="61"/>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
+      <c r="I11" s="61"/>
+      <c r="J11" s="61"/>
+      <c r="K11" s="93"/>
+      <c r="L11" s="94"/>
+      <c r="M11" s="94"/>
+      <c r="N11" s="94"/>
+      <c r="O11" s="94"/>
+      <c r="P11" s="94"/>
+      <c r="Q11" s="94"/>
+      <c r="R11" s="94"/>
+      <c r="S11" s="94"/>
+      <c r="T11" s="94"/>
+      <c r="U11" s="94"/>
+      <c r="V11" s="94"/>
+      <c r="W11" s="94"/>
+      <c r="X11" s="94"/>
+      <c r="Y11" s="94"/>
+      <c r="Z11" s="94"/>
     </row>
     <row r="12" ht="13.5" customHeight="1">
-      <c r="A12" s="94"/>
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="60"/>
-      <c r="I12" s="60"/>
-      <c r="J12" s="60"/>
-      <c r="K12" s="92"/>
-      <c r="L12" s="95"/>
-      <c r="M12" s="95"/>
-      <c r="N12" s="95"/>
-      <c r="O12" s="95"/>
-      <c r="P12" s="95"/>
-      <c r="Q12" s="95"/>
-      <c r="R12" s="95"/>
-      <c r="S12" s="95"/>
-      <c r="T12" s="95"/>
-      <c r="U12" s="95"/>
-      <c r="V12" s="95"/>
-      <c r="W12" s="95"/>
-      <c r="X12" s="95"/>
-      <c r="Y12" s="95"/>
-      <c r="Z12" s="95"/>
+      <c r="A12" s="112"/>
+      <c r="B12" s="61"/>
+      <c r="C12" s="61"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="61"/>
+      <c r="I12" s="61"/>
+      <c r="J12" s="61"/>
+      <c r="K12" s="93"/>
+      <c r="L12" s="96"/>
+      <c r="M12" s="96"/>
+      <c r="N12" s="96"/>
+      <c r="O12" s="96"/>
+      <c r="P12" s="96"/>
+      <c r="Q12" s="96"/>
+      <c r="R12" s="96"/>
+      <c r="S12" s="96"/>
+      <c r="T12" s="96"/>
+      <c r="U12" s="96"/>
+      <c r="V12" s="96"/>
+      <c r="W12" s="96"/>
+      <c r="X12" s="96"/>
+      <c r="Y12" s="96"/>
+      <c r="Z12" s="96"/>
     </row>
     <row r="13" ht="13.5" customHeight="1" outlineLevel="1">
-      <c r="A13" s="96"/>
-      <c r="B13" s="97"/>
-      <c r="C13" s="98"/>
-      <c r="D13" s="99"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="100"/>
-      <c r="H13" s="101"/>
-      <c r="I13" s="102"/>
-      <c r="J13" s="98" t="s">
-        <v>25</v>
+      <c r="A13" s="113"/>
+      <c r="B13" s="114"/>
+      <c r="C13" s="104"/>
+      <c r="D13" s="107"/>
+      <c r="E13" s="61"/>
+      <c r="F13" s="61"/>
+      <c r="G13" s="101"/>
+      <c r="H13" s="108"/>
+      <c r="I13" s="103"/>
+      <c r="J13" s="104" t="s">
+        <v>27</v>
       </c>
-      <c r="K13" s="98"/>
-      <c r="L13" s="95"/>
-      <c r="M13" s="95"/>
-      <c r="N13" s="95"/>
-      <c r="O13" s="95"/>
-      <c r="P13" s="95"/>
-      <c r="Q13" s="95"/>
-      <c r="R13" s="95"/>
-      <c r="S13" s="95"/>
-      <c r="T13" s="95"/>
-      <c r="U13" s="95"/>
-      <c r="V13" s="95"/>
-      <c r="W13" s="95"/>
-      <c r="X13" s="95"/>
-      <c r="Y13" s="95"/>
-      <c r="Z13" s="95"/>
+      <c r="K13" s="104"/>
+      <c r="L13" s="96"/>
+      <c r="M13" s="96"/>
+      <c r="N13" s="96"/>
+      <c r="O13" s="96"/>
+      <c r="P13" s="96"/>
+      <c r="Q13" s="96"/>
+      <c r="R13" s="96"/>
+      <c r="S13" s="96"/>
+      <c r="T13" s="96"/>
+      <c r="U13" s="96"/>
+      <c r="V13" s="96"/>
+      <c r="W13" s="96"/>
+      <c r="X13" s="96"/>
+      <c r="Y13" s="96"/>
+      <c r="Z13" s="96"/>
     </row>
     <row r="14" ht="13.5" customHeight="1" outlineLevel="1">
-      <c r="A14" s="103"/>
-      <c r="B14" s="60"/>
-      <c r="C14" s="104"/>
-      <c r="D14" s="105"/>
-      <c r="E14" s="105"/>
-      <c r="F14" s="105"/>
-      <c r="G14" s="105"/>
-      <c r="H14" s="105"/>
-      <c r="I14" s="105"/>
-      <c r="J14" s="105"/>
-      <c r="K14" s="106"/>
-      <c r="L14" s="95"/>
-      <c r="M14" s="95"/>
-      <c r="N14" s="95"/>
-      <c r="O14" s="95"/>
-      <c r="P14" s="95"/>
-      <c r="Q14" s="95"/>
-      <c r="R14" s="95"/>
-      <c r="S14" s="95"/>
-      <c r="T14" s="95"/>
-      <c r="U14" s="95"/>
-      <c r="V14" s="95"/>
-      <c r="W14" s="95"/>
-      <c r="X14" s="95"/>
-      <c r="Y14" s="95"/>
-      <c r="Z14" s="95"/>
+      <c r="A14" s="115"/>
+      <c r="B14" s="61"/>
+      <c r="C14" s="116"/>
+      <c r="D14" s="117"/>
+      <c r="E14" s="117"/>
+      <c r="F14" s="117"/>
+      <c r="G14" s="117"/>
+      <c r="H14" s="117"/>
+      <c r="I14" s="117"/>
+      <c r="J14" s="117"/>
+      <c r="K14" s="118"/>
+      <c r="L14" s="96"/>
+      <c r="M14" s="96"/>
+      <c r="N14" s="96"/>
+      <c r="O14" s="96"/>
+      <c r="P14" s="96"/>
+      <c r="Q14" s="96"/>
+      <c r="R14" s="96"/>
+      <c r="S14" s="96"/>
+      <c r="T14" s="96"/>
+      <c r="U14" s="96"/>
+      <c r="V14" s="96"/>
+      <c r="W14" s="96"/>
+      <c r="X14" s="96"/>
+      <c r="Y14" s="96"/>
+      <c r="Z14" s="96"/>
     </row>
     <row r="15" ht="63.75" customHeight="1" outlineLevel="1">
-      <c r="A15" s="96"/>
-      <c r="B15" s="107"/>
-      <c r="C15" s="108"/>
-      <c r="D15" s="109"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="60"/>
-      <c r="G15" s="100"/>
-      <c r="H15" s="101"/>
-      <c r="I15" s="99"/>
-      <c r="J15" s="98" t="s">
-        <v>25</v>
+      <c r="A15" s="113"/>
+      <c r="B15" s="119"/>
+      <c r="C15" s="120"/>
+      <c r="D15" s="121"/>
+      <c r="E15" s="61"/>
+      <c r="F15" s="61"/>
+      <c r="G15" s="101"/>
+      <c r="H15" s="108"/>
+      <c r="I15" s="107"/>
+      <c r="J15" s="104" t="s">
+        <v>27</v>
       </c>
-      <c r="K15" s="98"/>
-      <c r="L15" s="95"/>
-      <c r="M15" s="95"/>
-      <c r="N15" s="95"/>
-      <c r="O15" s="95"/>
-      <c r="P15" s="95"/>
-      <c r="Q15" s="95"/>
-      <c r="R15" s="95"/>
-      <c r="S15" s="95"/>
-      <c r="T15" s="95"/>
-      <c r="U15" s="95"/>
-      <c r="V15" s="95"/>
-      <c r="W15" s="95"/>
-      <c r="X15" s="95"/>
-      <c r="Y15" s="95"/>
-      <c r="Z15" s="95"/>
+      <c r="K15" s="104"/>
+      <c r="L15" s="96"/>
+      <c r="M15" s="96"/>
+      <c r="N15" s="96"/>
+      <c r="O15" s="96"/>
+      <c r="P15" s="96"/>
+      <c r="Q15" s="96"/>
+      <c r="R15" s="96"/>
+      <c r="S15" s="96"/>
+      <c r="T15" s="96"/>
+      <c r="U15" s="96"/>
+      <c r="V15" s="96"/>
+      <c r="W15" s="96"/>
+      <c r="X15" s="96"/>
+      <c r="Y15" s="96"/>
+      <c r="Z15" s="96"/>
     </row>
     <row r="16" ht="13.5" customHeight="1" outlineLevel="1">
-      <c r="A16" s="103"/>
-      <c r="B16" s="60"/>
-      <c r="C16" s="104"/>
-      <c r="D16" s="105"/>
-      <c r="E16" s="105"/>
-      <c r="F16" s="105"/>
-      <c r="G16" s="105"/>
-      <c r="H16" s="105"/>
-      <c r="I16" s="105"/>
-      <c r="J16" s="105"/>
-      <c r="K16" s="106"/>
-      <c r="L16" s="95"/>
-      <c r="M16" s="95"/>
-      <c r="N16" s="95"/>
-      <c r="O16" s="95"/>
-      <c r="P16" s="95"/>
-      <c r="Q16" s="95"/>
-      <c r="R16" s="95"/>
-      <c r="S16" s="95"/>
-      <c r="T16" s="95"/>
-      <c r="U16" s="95"/>
-      <c r="V16" s="95"/>
-      <c r="W16" s="95"/>
-      <c r="X16" s="95"/>
-      <c r="Y16" s="95"/>
-      <c r="Z16" s="95"/>
+      <c r="A16" s="115"/>
+      <c r="B16" s="61"/>
+      <c r="C16" s="116"/>
+      <c r="D16" s="117"/>
+      <c r="E16" s="117"/>
+      <c r="F16" s="117"/>
+      <c r="G16" s="117"/>
+      <c r="H16" s="117"/>
+      <c r="I16" s="117"/>
+      <c r="J16" s="117"/>
+      <c r="K16" s="118"/>
+      <c r="L16" s="96"/>
+      <c r="M16" s="96"/>
+      <c r="N16" s="96"/>
+      <c r="O16" s="96"/>
+      <c r="P16" s="96"/>
+      <c r="Q16" s="96"/>
+      <c r="R16" s="96"/>
+      <c r="S16" s="96"/>
+      <c r="T16" s="96"/>
+      <c r="U16" s="96"/>
+      <c r="V16" s="96"/>
+      <c r="W16" s="96"/>
+      <c r="X16" s="96"/>
+      <c r="Y16" s="96"/>
+      <c r="Z16" s="96"/>
     </row>
     <row r="17" ht="63.75" customHeight="1" outlineLevel="1">
-      <c r="A17" s="96"/>
-      <c r="B17" s="110"/>
-      <c r="C17" s="98"/>
-      <c r="D17" s="109"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="60"/>
-      <c r="G17" s="100"/>
-      <c r="H17" s="101"/>
-      <c r="I17" s="99"/>
-      <c r="J17" s="98" t="s">
-        <v>25</v>
+      <c r="A17" s="113"/>
+      <c r="B17" s="122"/>
+      <c r="C17" s="104"/>
+      <c r="D17" s="121"/>
+      <c r="E17" s="61"/>
+      <c r="F17" s="61"/>
+      <c r="G17" s="101"/>
+      <c r="H17" s="108"/>
+      <c r="I17" s="107"/>
+      <c r="J17" s="104" t="s">
+        <v>27</v>
       </c>
-      <c r="K17" s="98"/>
-      <c r="L17" s="95"/>
-      <c r="M17" s="95"/>
-      <c r="N17" s="95"/>
-      <c r="O17" s="95"/>
-      <c r="P17" s="95"/>
-      <c r="Q17" s="95"/>
-      <c r="R17" s="95"/>
-      <c r="S17" s="95"/>
-      <c r="T17" s="95"/>
-      <c r="U17" s="95"/>
-      <c r="V17" s="95"/>
-      <c r="W17" s="95"/>
-      <c r="X17" s="95"/>
-      <c r="Y17" s="95"/>
-      <c r="Z17" s="95"/>
+      <c r="K17" s="104"/>
+      <c r="L17" s="96"/>
+      <c r="M17" s="96"/>
+      <c r="N17" s="96"/>
+      <c r="O17" s="96"/>
+      <c r="P17" s="96"/>
+      <c r="Q17" s="96"/>
+      <c r="R17" s="96"/>
+      <c r="S17" s="96"/>
+      <c r="T17" s="96"/>
+      <c r="U17" s="96"/>
+      <c r="V17" s="96"/>
+      <c r="W17" s="96"/>
+      <c r="X17" s="96"/>
+      <c r="Y17" s="96"/>
+      <c r="Z17" s="96"/>
     </row>
     <row r="18" ht="12.0" customHeight="1">
       <c r="J18" s="11"/>
@@ -36779,477 +37052,477 @@
     </row>
     <row r="3" ht="15.0" customHeight="1">
       <c r="A3" s="51" t="s">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="C3" s="9"/>
       <c r="D3" s="10"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="53"/>
-      <c r="J3" s="54"/>
-      <c r="K3" s="55"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="57"/>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="57"/>
-      <c r="W3" s="57"/>
-      <c r="X3" s="57"/>
-      <c r="Y3" s="57"/>
-      <c r="Z3" s="57"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="53"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
+      <c r="L3" s="57"/>
+      <c r="M3" s="58"/>
+      <c r="N3" s="58"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="58"/>
+      <c r="Q3" s="58"/>
+      <c r="R3" s="58"/>
+      <c r="S3" s="58"/>
+      <c r="T3" s="58"/>
+      <c r="U3" s="58"/>
+      <c r="V3" s="58"/>
+      <c r="W3" s="58"/>
+      <c r="X3" s="58"/>
+      <c r="Y3" s="58"/>
+      <c r="Z3" s="58"/>
     </row>
     <row r="4" ht="13.5" customHeight="1">
-      <c r="A4" s="58" t="s">
-        <v>40</v>
+      <c r="A4" s="59" t="s">
+        <v>63</v>
       </c>
-      <c r="B4" s="59" t="s">
-        <v>22</v>
+      <c r="B4" s="110" t="s">
+        <v>60</v>
       </c>
-      <c r="C4" s="60"/>
-      <c r="D4" s="61"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="52"/>
-      <c r="I4" s="53"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="55"/>
-      <c r="L4" s="56"/>
-      <c r="M4" s="57"/>
-      <c r="N4" s="57"/>
-      <c r="O4" s="57"/>
-      <c r="P4" s="57"/>
-      <c r="Q4" s="57"/>
-      <c r="R4" s="57"/>
-      <c r="S4" s="57"/>
-      <c r="T4" s="57"/>
-      <c r="U4" s="57"/>
-      <c r="V4" s="57"/>
-      <c r="W4" s="57"/>
-      <c r="X4" s="57"/>
-      <c r="Y4" s="57"/>
-      <c r="Z4" s="57"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="56"/>
+      <c r="L4" s="57"/>
+      <c r="M4" s="58"/>
+      <c r="N4" s="58"/>
+      <c r="O4" s="58"/>
+      <c r="P4" s="58"/>
+      <c r="Q4" s="58"/>
+      <c r="R4" s="58"/>
+      <c r="S4" s="58"/>
+      <c r="T4" s="58"/>
+      <c r="U4" s="58"/>
+      <c r="V4" s="58"/>
+      <c r="W4" s="58"/>
+      <c r="X4" s="58"/>
+      <c r="Y4" s="58"/>
+      <c r="Z4" s="58"/>
     </row>
     <row r="5" ht="13.5" customHeight="1">
-      <c r="A5" s="58" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="62" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="60"/>
-      <c r="D5" s="61"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
-      <c r="I5" s="64"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="55"/>
-      <c r="L5" s="65"/>
-      <c r="M5" s="66"/>
-      <c r="N5" s="66"/>
-      <c r="O5" s="66"/>
-      <c r="P5" s="66"/>
-      <c r="Q5" s="66"/>
-      <c r="R5" s="66"/>
-      <c r="S5" s="66"/>
-      <c r="T5" s="66"/>
-      <c r="U5" s="66"/>
-      <c r="V5" s="66"/>
-      <c r="W5" s="66"/>
-      <c r="X5" s="66"/>
-      <c r="Y5" s="66"/>
-      <c r="Z5" s="66"/>
-    </row>
-    <row r="6" ht="15.0" customHeight="1">
-      <c r="A6" s="67" t="s">
+      <c r="A5" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="68">
+      <c r="B5" s="111" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="61"/>
+      <c r="D5" s="62"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="65"/>
+      <c r="J5" s="55"/>
+      <c r="K5" s="56"/>
+      <c r="L5" s="66"/>
+      <c r="M5" s="67"/>
+      <c r="N5" s="67"/>
+      <c r="O5" s="67"/>
+      <c r="P5" s="67"/>
+      <c r="Q5" s="67"/>
+      <c r="R5" s="67"/>
+      <c r="S5" s="67"/>
+      <c r="T5" s="67"/>
+      <c r="U5" s="67"/>
+      <c r="V5" s="67"/>
+      <c r="W5" s="67"/>
+      <c r="X5" s="67"/>
+      <c r="Y5" s="67"/>
+      <c r="Z5" s="67"/>
+    </row>
+    <row r="6" ht="15.0" customHeight="1">
+      <c r="A6" s="68" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="69">
         <f>COUNTIF(J12:J17,"Pass")</f>
         <v>3</v>
       </c>
-      <c r="C6" s="69" t="s">
-        <v>26</v>
+      <c r="C6" s="70" t="s">
+        <v>28</v>
       </c>
-      <c r="D6" s="70">
+      <c r="D6" s="71">
         <f>COUNTIF(J10:J736,"Pending")</f>
         <v>0</v>
       </c>
-      <c r="E6" s="71"/>
-      <c r="F6" s="71"/>
-      <c r="G6" s="71"/>
-      <c r="H6" s="71"/>
-      <c r="I6" s="53"/>
-      <c r="J6" s="54"/>
-      <c r="K6" s="55"/>
-      <c r="L6" s="56"/>
-      <c r="M6" s="57"/>
-      <c r="N6" s="57"/>
-      <c r="O6" s="57"/>
-      <c r="P6" s="57"/>
-      <c r="Q6" s="57"/>
-      <c r="R6" s="57"/>
-      <c r="S6" s="57"/>
-      <c r="T6" s="57"/>
-      <c r="U6" s="57"/>
-      <c r="V6" s="57"/>
-      <c r="W6" s="57"/>
-      <c r="X6" s="57"/>
-      <c r="Y6" s="57"/>
-      <c r="Z6" s="57"/>
+      <c r="E6" s="72"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="72"/>
+      <c r="H6" s="72"/>
+      <c r="I6" s="54"/>
+      <c r="J6" s="55"/>
+      <c r="K6" s="56"/>
+      <c r="L6" s="57"/>
+      <c r="M6" s="58"/>
+      <c r="N6" s="58"/>
+      <c r="O6" s="58"/>
+      <c r="P6" s="58"/>
+      <c r="Q6" s="58"/>
+      <c r="R6" s="58"/>
+      <c r="S6" s="58"/>
+      <c r="T6" s="58"/>
+      <c r="U6" s="58"/>
+      <c r="V6" s="58"/>
+      <c r="W6" s="58"/>
+      <c r="X6" s="58"/>
+      <c r="Y6" s="58"/>
+      <c r="Z6" s="58"/>
     </row>
     <row r="7" ht="15.0" customHeight="1">
-      <c r="A7" s="72" t="s">
-        <v>27</v>
+      <c r="A7" s="73" t="s">
+        <v>29</v>
       </c>
-      <c r="B7" s="73">
+      <c r="B7" s="74">
         <f>COUNTIF(J12:J17,"Fail")</f>
         <v>0</v>
       </c>
-      <c r="C7" s="74" t="s">
-        <v>28</v>
+      <c r="C7" s="75" t="s">
+        <v>30</v>
       </c>
-      <c r="D7" s="75">
+      <c r="D7" s="76">
         <f>COUNTA(A12:A17) -15</f>
         <v>-15</v>
       </c>
-      <c r="E7" s="76"/>
-      <c r="F7" s="76"/>
-      <c r="G7" s="76"/>
-      <c r="H7" s="76"/>
-      <c r="I7" s="53"/>
-      <c r="J7" s="54"/>
-      <c r="K7" s="55"/>
-      <c r="L7" s="56"/>
-      <c r="M7" s="57"/>
-      <c r="N7" s="57"/>
-      <c r="O7" s="57"/>
-      <c r="P7" s="57"/>
-      <c r="Q7" s="57"/>
-      <c r="R7" s="57"/>
-      <c r="S7" s="57"/>
-      <c r="T7" s="57"/>
-      <c r="U7" s="57"/>
-      <c r="V7" s="57"/>
-      <c r="W7" s="57"/>
-      <c r="X7" s="57"/>
-      <c r="Y7" s="57"/>
-      <c r="Z7" s="57"/>
+      <c r="E7" s="77"/>
+      <c r="F7" s="77"/>
+      <c r="G7" s="77"/>
+      <c r="H7" s="77"/>
+      <c r="I7" s="54"/>
+      <c r="J7" s="55"/>
+      <c r="K7" s="56"/>
+      <c r="L7" s="57"/>
+      <c r="M7" s="58"/>
+      <c r="N7" s="58"/>
+      <c r="O7" s="58"/>
+      <c r="P7" s="58"/>
+      <c r="Q7" s="58"/>
+      <c r="R7" s="58"/>
+      <c r="S7" s="58"/>
+      <c r="T7" s="58"/>
+      <c r="U7" s="58"/>
+      <c r="V7" s="58"/>
+      <c r="W7" s="58"/>
+      <c r="X7" s="58"/>
+      <c r="Y7" s="58"/>
+      <c r="Z7" s="58"/>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="77"/>
+      <c r="A8" s="78"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
-      <c r="D8" s="78"/>
-      <c r="E8" s="71"/>
-      <c r="F8" s="71"/>
-      <c r="G8" s="71"/>
-      <c r="H8" s="71"/>
-      <c r="I8" s="71"/>
-      <c r="J8" s="79"/>
-      <c r="K8" s="79"/>
-      <c r="L8" s="56"/>
-      <c r="M8" s="57"/>
-      <c r="N8" s="57"/>
-      <c r="O8" s="57"/>
-      <c r="P8" s="57"/>
-      <c r="Q8" s="57"/>
-      <c r="R8" s="57"/>
-      <c r="S8" s="57"/>
-      <c r="T8" s="57"/>
-      <c r="U8" s="57"/>
-      <c r="V8" s="57"/>
-      <c r="W8" s="57"/>
-      <c r="X8" s="57"/>
-      <c r="Y8" s="57"/>
-      <c r="Z8" s="57"/>
+      <c r="D8" s="79"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="72"/>
+      <c r="H8" s="72"/>
+      <c r="I8" s="72"/>
+      <c r="J8" s="80"/>
+      <c r="K8" s="80"/>
+      <c r="L8" s="57"/>
+      <c r="M8" s="58"/>
+      <c r="N8" s="58"/>
+      <c r="O8" s="58"/>
+      <c r="P8" s="58"/>
+      <c r="Q8" s="58"/>
+      <c r="R8" s="58"/>
+      <c r="S8" s="58"/>
+      <c r="T8" s="58"/>
+      <c r="U8" s="58"/>
+      <c r="V8" s="58"/>
+      <c r="W8" s="58"/>
+      <c r="X8" s="58"/>
+      <c r="Y8" s="58"/>
+      <c r="Z8" s="58"/>
     </row>
     <row r="9" ht="12.0" customHeight="1">
-      <c r="A9" s="80" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="81" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="80" t="s">
+      <c r="A9" s="81" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="82" t="s">
+      <c r="B9" s="82" t="s">
         <v>32</v>
+      </c>
+      <c r="C9" s="81" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="83" t="s">
+        <v>34</v>
       </c>
       <c r="E9" s="42"/>
       <c r="F9" s="42"/>
-      <c r="G9" s="83"/>
-      <c r="H9" s="80" t="s">
-        <v>33</v>
-      </c>
-      <c r="I9" s="84" t="s">
-        <v>34</v>
-      </c>
-      <c r="J9" s="84" t="s">
+      <c r="G9" s="84"/>
+      <c r="H9" s="81" t="s">
         <v>35</v>
       </c>
-      <c r="K9" s="84" t="s">
+      <c r="I9" s="85" t="s">
         <v>36</v>
       </c>
-      <c r="L9" s="85"/>
-      <c r="M9" s="86"/>
-      <c r="N9" s="86"/>
-      <c r="O9" s="86"/>
-      <c r="P9" s="86"/>
-      <c r="Q9" s="86"/>
-      <c r="R9" s="86"/>
-      <c r="S9" s="86"/>
-      <c r="T9" s="86"/>
-      <c r="U9" s="86"/>
-      <c r="V9" s="86"/>
-      <c r="W9" s="86"/>
-      <c r="X9" s="86"/>
-      <c r="Y9" s="86"/>
-      <c r="Z9" s="86"/>
+      <c r="J9" s="85" t="s">
+        <v>37</v>
+      </c>
+      <c r="K9" s="85" t="s">
+        <v>38</v>
+      </c>
+      <c r="L9" s="86"/>
+      <c r="M9" s="87"/>
+      <c r="N9" s="87"/>
+      <c r="O9" s="87"/>
+      <c r="P9" s="87"/>
+      <c r="Q9" s="87"/>
+      <c r="R9" s="87"/>
+      <c r="S9" s="87"/>
+      <c r="T9" s="87"/>
+      <c r="U9" s="87"/>
+      <c r="V9" s="87"/>
+      <c r="W9" s="87"/>
+      <c r="X9" s="87"/>
+      <c r="Y9" s="87"/>
+      <c r="Z9" s="87"/>
     </row>
     <row r="10" ht="12.0" customHeight="1">
-      <c r="A10" s="87"/>
-      <c r="B10" s="87"/>
-      <c r="C10" s="87"/>
-      <c r="D10" s="88"/>
-      <c r="E10" s="89"/>
-      <c r="F10" s="89"/>
-      <c r="G10" s="90"/>
-      <c r="H10" s="87"/>
-      <c r="I10" s="87"/>
-      <c r="J10" s="87"/>
-      <c r="K10" s="87"/>
-      <c r="L10" s="56"/>
-      <c r="M10" s="57"/>
-      <c r="N10" s="57"/>
-      <c r="O10" s="57"/>
-      <c r="P10" s="57"/>
-      <c r="Q10" s="57"/>
-      <c r="R10" s="57"/>
-      <c r="S10" s="57"/>
-      <c r="T10" s="57"/>
-      <c r="U10" s="57"/>
-      <c r="V10" s="57"/>
-      <c r="W10" s="57"/>
-      <c r="X10" s="57"/>
-      <c r="Y10" s="57"/>
-      <c r="Z10" s="57"/>
+      <c r="A10" s="88"/>
+      <c r="B10" s="88"/>
+      <c r="C10" s="88"/>
+      <c r="D10" s="89"/>
+      <c r="E10" s="90"/>
+      <c r="F10" s="90"/>
+      <c r="G10" s="91"/>
+      <c r="H10" s="88"/>
+      <c r="I10" s="88"/>
+      <c r="J10" s="88"/>
+      <c r="K10" s="88"/>
+      <c r="L10" s="57"/>
+      <c r="M10" s="58"/>
+      <c r="N10" s="58"/>
+      <c r="O10" s="58"/>
+      <c r="P10" s="58"/>
+      <c r="Q10" s="58"/>
+      <c r="R10" s="58"/>
+      <c r="S10" s="58"/>
+      <c r="T10" s="58"/>
+      <c r="U10" s="58"/>
+      <c r="V10" s="58"/>
+      <c r="W10" s="58"/>
+      <c r="X10" s="58"/>
+      <c r="Y10" s="58"/>
+      <c r="Z10" s="58"/>
     </row>
     <row r="11" ht="13.5" customHeight="1">
-      <c r="A11" s="91"/>
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
-      <c r="I11" s="60"/>
-      <c r="J11" s="60"/>
-      <c r="K11" s="92"/>
-      <c r="L11" s="93"/>
-      <c r="M11" s="93"/>
-      <c r="N11" s="93"/>
-      <c r="O11" s="93"/>
-      <c r="P11" s="93"/>
-      <c r="Q11" s="93"/>
-      <c r="R11" s="93"/>
-      <c r="S11" s="93"/>
-      <c r="T11" s="93"/>
-      <c r="U11" s="93"/>
-      <c r="V11" s="93"/>
-      <c r="W11" s="93"/>
-      <c r="X11" s="93"/>
-      <c r="Y11" s="93"/>
-      <c r="Z11" s="93"/>
+      <c r="A11" s="92"/>
+      <c r="B11" s="61"/>
+      <c r="C11" s="61"/>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
+      <c r="I11" s="61"/>
+      <c r="J11" s="61"/>
+      <c r="K11" s="93"/>
+      <c r="L11" s="94"/>
+      <c r="M11" s="94"/>
+      <c r="N11" s="94"/>
+      <c r="O11" s="94"/>
+      <c r="P11" s="94"/>
+      <c r="Q11" s="94"/>
+      <c r="R11" s="94"/>
+      <c r="S11" s="94"/>
+      <c r="T11" s="94"/>
+      <c r="U11" s="94"/>
+      <c r="V11" s="94"/>
+      <c r="W11" s="94"/>
+      <c r="X11" s="94"/>
+      <c r="Y11" s="94"/>
+      <c r="Z11" s="94"/>
     </row>
     <row r="12" ht="13.5" customHeight="1">
-      <c r="A12" s="94"/>
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="60"/>
-      <c r="I12" s="60"/>
-      <c r="J12" s="60"/>
-      <c r="K12" s="92"/>
-      <c r="L12" s="95"/>
-      <c r="M12" s="95"/>
-      <c r="N12" s="95"/>
-      <c r="O12" s="95"/>
-      <c r="P12" s="95"/>
-      <c r="Q12" s="95"/>
-      <c r="R12" s="95"/>
-      <c r="S12" s="95"/>
-      <c r="T12" s="95"/>
-      <c r="U12" s="95"/>
-      <c r="V12" s="95"/>
-      <c r="W12" s="95"/>
-      <c r="X12" s="95"/>
-      <c r="Y12" s="95"/>
-      <c r="Z12" s="95"/>
+      <c r="A12" s="112"/>
+      <c r="B12" s="61"/>
+      <c r="C12" s="61"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="61"/>
+      <c r="I12" s="61"/>
+      <c r="J12" s="61"/>
+      <c r="K12" s="93"/>
+      <c r="L12" s="96"/>
+      <c r="M12" s="96"/>
+      <c r="N12" s="96"/>
+      <c r="O12" s="96"/>
+      <c r="P12" s="96"/>
+      <c r="Q12" s="96"/>
+      <c r="R12" s="96"/>
+      <c r="S12" s="96"/>
+      <c r="T12" s="96"/>
+      <c r="U12" s="96"/>
+      <c r="V12" s="96"/>
+      <c r="W12" s="96"/>
+      <c r="X12" s="96"/>
+      <c r="Y12" s="96"/>
+      <c r="Z12" s="96"/>
     </row>
     <row r="13" ht="13.5" customHeight="1" outlineLevel="1">
-      <c r="A13" s="96"/>
-      <c r="B13" s="97"/>
-      <c r="C13" s="98"/>
-      <c r="D13" s="99"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="100"/>
-      <c r="H13" s="101"/>
-      <c r="I13" s="102"/>
-      <c r="J13" s="98" t="s">
-        <v>25</v>
+      <c r="A13" s="113"/>
+      <c r="B13" s="114"/>
+      <c r="C13" s="104"/>
+      <c r="D13" s="107"/>
+      <c r="E13" s="61"/>
+      <c r="F13" s="61"/>
+      <c r="G13" s="101"/>
+      <c r="H13" s="108"/>
+      <c r="I13" s="103"/>
+      <c r="J13" s="104" t="s">
+        <v>27</v>
       </c>
-      <c r="K13" s="98"/>
-      <c r="L13" s="95"/>
-      <c r="M13" s="95"/>
-      <c r="N13" s="95"/>
-      <c r="O13" s="95"/>
-      <c r="P13" s="95"/>
-      <c r="Q13" s="95"/>
-      <c r="R13" s="95"/>
-      <c r="S13" s="95"/>
-      <c r="T13" s="95"/>
-      <c r="U13" s="95"/>
-      <c r="V13" s="95"/>
-      <c r="W13" s="95"/>
-      <c r="X13" s="95"/>
-      <c r="Y13" s="95"/>
-      <c r="Z13" s="95"/>
+      <c r="K13" s="104"/>
+      <c r="L13" s="96"/>
+      <c r="M13" s="96"/>
+      <c r="N13" s="96"/>
+      <c r="O13" s="96"/>
+      <c r="P13" s="96"/>
+      <c r="Q13" s="96"/>
+      <c r="R13" s="96"/>
+      <c r="S13" s="96"/>
+      <c r="T13" s="96"/>
+      <c r="U13" s="96"/>
+      <c r="V13" s="96"/>
+      <c r="W13" s="96"/>
+      <c r="X13" s="96"/>
+      <c r="Y13" s="96"/>
+      <c r="Z13" s="96"/>
     </row>
     <row r="14" ht="13.5" customHeight="1" outlineLevel="1">
-      <c r="A14" s="103"/>
-      <c r="B14" s="60"/>
-      <c r="C14" s="104"/>
-      <c r="D14" s="105"/>
-      <c r="E14" s="105"/>
-      <c r="F14" s="105"/>
-      <c r="G14" s="105"/>
-      <c r="H14" s="105"/>
-      <c r="I14" s="105"/>
-      <c r="J14" s="105"/>
-      <c r="K14" s="106"/>
-      <c r="L14" s="95"/>
-      <c r="M14" s="95"/>
-      <c r="N14" s="95"/>
-      <c r="O14" s="95"/>
-      <c r="P14" s="95"/>
-      <c r="Q14" s="95"/>
-      <c r="R14" s="95"/>
-      <c r="S14" s="95"/>
-      <c r="T14" s="95"/>
-      <c r="U14" s="95"/>
-      <c r="V14" s="95"/>
-      <c r="W14" s="95"/>
-      <c r="X14" s="95"/>
-      <c r="Y14" s="95"/>
-      <c r="Z14" s="95"/>
+      <c r="A14" s="115"/>
+      <c r="B14" s="61"/>
+      <c r="C14" s="116"/>
+      <c r="D14" s="117"/>
+      <c r="E14" s="117"/>
+      <c r="F14" s="117"/>
+      <c r="G14" s="117"/>
+      <c r="H14" s="117"/>
+      <c r="I14" s="117"/>
+      <c r="J14" s="117"/>
+      <c r="K14" s="118"/>
+      <c r="L14" s="96"/>
+      <c r="M14" s="96"/>
+      <c r="N14" s="96"/>
+      <c r="O14" s="96"/>
+      <c r="P14" s="96"/>
+      <c r="Q14" s="96"/>
+      <c r="R14" s="96"/>
+      <c r="S14" s="96"/>
+      <c r="T14" s="96"/>
+      <c r="U14" s="96"/>
+      <c r="V14" s="96"/>
+      <c r="W14" s="96"/>
+      <c r="X14" s="96"/>
+      <c r="Y14" s="96"/>
+      <c r="Z14" s="96"/>
     </row>
     <row r="15" ht="63.75" customHeight="1" outlineLevel="1">
-      <c r="A15" s="96"/>
-      <c r="B15" s="107"/>
-      <c r="C15" s="108"/>
-      <c r="D15" s="109"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="60"/>
-      <c r="G15" s="100"/>
-      <c r="H15" s="101"/>
-      <c r="I15" s="99"/>
-      <c r="J15" s="98" t="s">
-        <v>25</v>
+      <c r="A15" s="113"/>
+      <c r="B15" s="119"/>
+      <c r="C15" s="120"/>
+      <c r="D15" s="121"/>
+      <c r="E15" s="61"/>
+      <c r="F15" s="61"/>
+      <c r="G15" s="101"/>
+      <c r="H15" s="108"/>
+      <c r="I15" s="107"/>
+      <c r="J15" s="104" t="s">
+        <v>27</v>
       </c>
-      <c r="K15" s="98"/>
-      <c r="L15" s="95"/>
-      <c r="M15" s="95"/>
-      <c r="N15" s="95"/>
-      <c r="O15" s="95"/>
-      <c r="P15" s="95"/>
-      <c r="Q15" s="95"/>
-      <c r="R15" s="95"/>
-      <c r="S15" s="95"/>
-      <c r="T15" s="95"/>
-      <c r="U15" s="95"/>
-      <c r="V15" s="95"/>
-      <c r="W15" s="95"/>
-      <c r="X15" s="95"/>
-      <c r="Y15" s="95"/>
-      <c r="Z15" s="95"/>
+      <c r="K15" s="104"/>
+      <c r="L15" s="96"/>
+      <c r="M15" s="96"/>
+      <c r="N15" s="96"/>
+      <c r="O15" s="96"/>
+      <c r="P15" s="96"/>
+      <c r="Q15" s="96"/>
+      <c r="R15" s="96"/>
+      <c r="S15" s="96"/>
+      <c r="T15" s="96"/>
+      <c r="U15" s="96"/>
+      <c r="V15" s="96"/>
+      <c r="W15" s="96"/>
+      <c r="X15" s="96"/>
+      <c r="Y15" s="96"/>
+      <c r="Z15" s="96"/>
     </row>
     <row r="16" ht="13.5" customHeight="1" outlineLevel="1">
-      <c r="A16" s="103"/>
-      <c r="B16" s="60"/>
-      <c r="C16" s="104"/>
-      <c r="D16" s="105"/>
-      <c r="E16" s="105"/>
-      <c r="F16" s="105"/>
-      <c r="G16" s="105"/>
-      <c r="H16" s="105"/>
-      <c r="I16" s="105"/>
-      <c r="J16" s="105"/>
-      <c r="K16" s="106"/>
-      <c r="L16" s="95"/>
-      <c r="M16" s="95"/>
-      <c r="N16" s="95"/>
-      <c r="O16" s="95"/>
-      <c r="P16" s="95"/>
-      <c r="Q16" s="95"/>
-      <c r="R16" s="95"/>
-      <c r="S16" s="95"/>
-      <c r="T16" s="95"/>
-      <c r="U16" s="95"/>
-      <c r="V16" s="95"/>
-      <c r="W16" s="95"/>
-      <c r="X16" s="95"/>
-      <c r="Y16" s="95"/>
-      <c r="Z16" s="95"/>
+      <c r="A16" s="115"/>
+      <c r="B16" s="61"/>
+      <c r="C16" s="116"/>
+      <c r="D16" s="117"/>
+      <c r="E16" s="117"/>
+      <c r="F16" s="117"/>
+      <c r="G16" s="117"/>
+      <c r="H16" s="117"/>
+      <c r="I16" s="117"/>
+      <c r="J16" s="117"/>
+      <c r="K16" s="118"/>
+      <c r="L16" s="96"/>
+      <c r="M16" s="96"/>
+      <c r="N16" s="96"/>
+      <c r="O16" s="96"/>
+      <c r="P16" s="96"/>
+      <c r="Q16" s="96"/>
+      <c r="R16" s="96"/>
+      <c r="S16" s="96"/>
+      <c r="T16" s="96"/>
+      <c r="U16" s="96"/>
+      <c r="V16" s="96"/>
+      <c r="W16" s="96"/>
+      <c r="X16" s="96"/>
+      <c r="Y16" s="96"/>
+      <c r="Z16" s="96"/>
     </row>
     <row r="17" ht="63.75" customHeight="1" outlineLevel="1">
-      <c r="A17" s="96"/>
-      <c r="B17" s="110"/>
-      <c r="C17" s="98"/>
-      <c r="D17" s="109"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="60"/>
-      <c r="G17" s="100"/>
-      <c r="H17" s="101"/>
-      <c r="I17" s="99"/>
-      <c r="J17" s="98" t="s">
-        <v>25</v>
+      <c r="A17" s="113"/>
+      <c r="B17" s="122"/>
+      <c r="C17" s="104"/>
+      <c r="D17" s="121"/>
+      <c r="E17" s="61"/>
+      <c r="F17" s="61"/>
+      <c r="G17" s="101"/>
+      <c r="H17" s="108"/>
+      <c r="I17" s="107"/>
+      <c r="J17" s="104" t="s">
+        <v>27</v>
       </c>
-      <c r="K17" s="98"/>
-      <c r="L17" s="95"/>
-      <c r="M17" s="95"/>
-      <c r="N17" s="95"/>
-      <c r="O17" s="95"/>
-      <c r="P17" s="95"/>
-      <c r="Q17" s="95"/>
-      <c r="R17" s="95"/>
-      <c r="S17" s="95"/>
-      <c r="T17" s="95"/>
-      <c r="U17" s="95"/>
-      <c r="V17" s="95"/>
-      <c r="W17" s="95"/>
-      <c r="X17" s="95"/>
-      <c r="Y17" s="95"/>
-      <c r="Z17" s="95"/>
+      <c r="K17" s="104"/>
+      <c r="L17" s="96"/>
+      <c r="M17" s="96"/>
+      <c r="N17" s="96"/>
+      <c r="O17" s="96"/>
+      <c r="P17" s="96"/>
+      <c r="Q17" s="96"/>
+      <c r="R17" s="96"/>
+      <c r="S17" s="96"/>
+      <c r="T17" s="96"/>
+      <c r="U17" s="96"/>
+      <c r="V17" s="96"/>
+      <c r="W17" s="96"/>
+      <c r="X17" s="96"/>
+      <c r="Y17" s="96"/>
+      <c r="Z17" s="96"/>
     </row>
     <row r="18" ht="12.0" customHeight="1">
       <c r="J18" s="11"/>
@@ -40316,477 +40589,477 @@
     </row>
     <row r="3" ht="15.0" customHeight="1">
       <c r="A3" s="51" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="C3" s="9"/>
       <c r="D3" s="10"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="53"/>
-      <c r="J3" s="54"/>
-      <c r="K3" s="55"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="57"/>
-      <c r="N3" s="57"/>
-      <c r="O3" s="57"/>
-      <c r="P3" s="57"/>
-      <c r="Q3" s="57"/>
-      <c r="R3" s="57"/>
-      <c r="S3" s="57"/>
-      <c r="T3" s="57"/>
-      <c r="U3" s="57"/>
-      <c r="V3" s="57"/>
-      <c r="W3" s="57"/>
-      <c r="X3" s="57"/>
-      <c r="Y3" s="57"/>
-      <c r="Z3" s="57"/>
+      <c r="E3" s="53"/>
+      <c r="F3" s="53"/>
+      <c r="G3" s="53"/>
+      <c r="H3" s="53"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="55"/>
+      <c r="K3" s="56"/>
+      <c r="L3" s="57"/>
+      <c r="M3" s="58"/>
+      <c r="N3" s="58"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="58"/>
+      <c r="Q3" s="58"/>
+      <c r="R3" s="58"/>
+      <c r="S3" s="58"/>
+      <c r="T3" s="58"/>
+      <c r="U3" s="58"/>
+      <c r="V3" s="58"/>
+      <c r="W3" s="58"/>
+      <c r="X3" s="58"/>
+      <c r="Y3" s="58"/>
+      <c r="Z3" s="58"/>
     </row>
     <row r="4" ht="13.5" customHeight="1">
-      <c r="A4" s="58" t="s">
-        <v>42</v>
+      <c r="A4" s="59" t="s">
+        <v>65</v>
       </c>
-      <c r="B4" s="59" t="s">
-        <v>22</v>
+      <c r="B4" s="110" t="s">
+        <v>60</v>
       </c>
-      <c r="C4" s="60"/>
-      <c r="D4" s="61"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="52"/>
-      <c r="I4" s="53"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="55"/>
-      <c r="L4" s="56"/>
-      <c r="M4" s="57"/>
-      <c r="N4" s="57"/>
-      <c r="O4" s="57"/>
-      <c r="P4" s="57"/>
-      <c r="Q4" s="57"/>
-      <c r="R4" s="57"/>
-      <c r="S4" s="57"/>
-      <c r="T4" s="57"/>
-      <c r="U4" s="57"/>
-      <c r="V4" s="57"/>
-      <c r="W4" s="57"/>
-      <c r="X4" s="57"/>
-      <c r="Y4" s="57"/>
-      <c r="Z4" s="57"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="53"/>
+      <c r="G4" s="53"/>
+      <c r="H4" s="53"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="55"/>
+      <c r="K4" s="56"/>
+      <c r="L4" s="57"/>
+      <c r="M4" s="58"/>
+      <c r="N4" s="58"/>
+      <c r="O4" s="58"/>
+      <c r="P4" s="58"/>
+      <c r="Q4" s="58"/>
+      <c r="R4" s="58"/>
+      <c r="S4" s="58"/>
+      <c r="T4" s="58"/>
+      <c r="U4" s="58"/>
+      <c r="V4" s="58"/>
+      <c r="W4" s="58"/>
+      <c r="X4" s="58"/>
+      <c r="Y4" s="58"/>
+      <c r="Z4" s="58"/>
     </row>
     <row r="5" ht="13.5" customHeight="1">
-      <c r="A5" s="58" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="62" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="60"/>
-      <c r="D5" s="61"/>
-      <c r="E5" s="63"/>
-      <c r="F5" s="63"/>
-      <c r="G5" s="63"/>
-      <c r="H5" s="63"/>
-      <c r="I5" s="64"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="55"/>
-      <c r="L5" s="65"/>
-      <c r="M5" s="66"/>
-      <c r="N5" s="66"/>
-      <c r="O5" s="66"/>
-      <c r="P5" s="66"/>
-      <c r="Q5" s="66"/>
-      <c r="R5" s="66"/>
-      <c r="S5" s="66"/>
-      <c r="T5" s="66"/>
-      <c r="U5" s="66"/>
-      <c r="V5" s="66"/>
-      <c r="W5" s="66"/>
-      <c r="X5" s="66"/>
-      <c r="Y5" s="66"/>
-      <c r="Z5" s="66"/>
-    </row>
-    <row r="6" ht="15.0" customHeight="1">
-      <c r="A6" s="67" t="s">
+      <c r="A5" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="68">
+      <c r="B5" s="111" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="61"/>
+      <c r="D5" s="62"/>
+      <c r="E5" s="64"/>
+      <c r="F5" s="64"/>
+      <c r="G5" s="64"/>
+      <c r="H5" s="64"/>
+      <c r="I5" s="65"/>
+      <c r="J5" s="55"/>
+      <c r="K5" s="56"/>
+      <c r="L5" s="66"/>
+      <c r="M5" s="67"/>
+      <c r="N5" s="67"/>
+      <c r="O5" s="67"/>
+      <c r="P5" s="67"/>
+      <c r="Q5" s="67"/>
+      <c r="R5" s="67"/>
+      <c r="S5" s="67"/>
+      <c r="T5" s="67"/>
+      <c r="U5" s="67"/>
+      <c r="V5" s="67"/>
+      <c r="W5" s="67"/>
+      <c r="X5" s="67"/>
+      <c r="Y5" s="67"/>
+      <c r="Z5" s="67"/>
+    </row>
+    <row r="6" ht="15.0" customHeight="1">
+      <c r="A6" s="68" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="69">
         <f>COUNTIF(J12:J17,"Pass")</f>
         <v>3</v>
       </c>
-      <c r="C6" s="69" t="s">
-        <v>26</v>
+      <c r="C6" s="70" t="s">
+        <v>28</v>
       </c>
-      <c r="D6" s="70">
+      <c r="D6" s="71">
         <f>COUNTIF(J10:J736,"Pending")</f>
         <v>0</v>
       </c>
-      <c r="E6" s="71"/>
-      <c r="F6" s="71"/>
-      <c r="G6" s="71"/>
-      <c r="H6" s="71"/>
-      <c r="I6" s="53"/>
-      <c r="J6" s="54"/>
-      <c r="K6" s="55"/>
-      <c r="L6" s="56"/>
-      <c r="M6" s="57"/>
-      <c r="N6" s="57"/>
-      <c r="O6" s="57"/>
-      <c r="P6" s="57"/>
-      <c r="Q6" s="57"/>
-      <c r="R6" s="57"/>
-      <c r="S6" s="57"/>
-      <c r="T6" s="57"/>
-      <c r="U6" s="57"/>
-      <c r="V6" s="57"/>
-      <c r="W6" s="57"/>
-      <c r="X6" s="57"/>
-      <c r="Y6" s="57"/>
-      <c r="Z6" s="57"/>
+      <c r="E6" s="72"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="72"/>
+      <c r="H6" s="72"/>
+      <c r="I6" s="54"/>
+      <c r="J6" s="55"/>
+      <c r="K6" s="56"/>
+      <c r="L6" s="57"/>
+      <c r="M6" s="58"/>
+      <c r="N6" s="58"/>
+      <c r="O6" s="58"/>
+      <c r="P6" s="58"/>
+      <c r="Q6" s="58"/>
+      <c r="R6" s="58"/>
+      <c r="S6" s="58"/>
+      <c r="T6" s="58"/>
+      <c r="U6" s="58"/>
+      <c r="V6" s="58"/>
+      <c r="W6" s="58"/>
+      <c r="X6" s="58"/>
+      <c r="Y6" s="58"/>
+      <c r="Z6" s="58"/>
     </row>
     <row r="7" ht="15.0" customHeight="1">
-      <c r="A7" s="72" t="s">
-        <v>27</v>
+      <c r="A7" s="73" t="s">
+        <v>29</v>
       </c>
-      <c r="B7" s="73">
+      <c r="B7" s="74">
         <f>COUNTIF(J12:J17,"Fail")</f>
         <v>0</v>
       </c>
-      <c r="C7" s="74" t="s">
-        <v>28</v>
+      <c r="C7" s="75" t="s">
+        <v>30</v>
       </c>
-      <c r="D7" s="75">
+      <c r="D7" s="76">
         <f>COUNTA(A12:A17) -15</f>
         <v>-15</v>
       </c>
-      <c r="E7" s="76"/>
-      <c r="F7" s="76"/>
-      <c r="G7" s="76"/>
-      <c r="H7" s="76"/>
-      <c r="I7" s="53"/>
-      <c r="J7" s="54"/>
-      <c r="K7" s="55"/>
-      <c r="L7" s="56"/>
-      <c r="M7" s="57"/>
-      <c r="N7" s="57"/>
-      <c r="O7" s="57"/>
-      <c r="P7" s="57"/>
-      <c r="Q7" s="57"/>
-      <c r="R7" s="57"/>
-      <c r="S7" s="57"/>
-      <c r="T7" s="57"/>
-      <c r="U7" s="57"/>
-      <c r="V7" s="57"/>
-      <c r="W7" s="57"/>
-      <c r="X7" s="57"/>
-      <c r="Y7" s="57"/>
-      <c r="Z7" s="57"/>
+      <c r="E7" s="77"/>
+      <c r="F7" s="77"/>
+      <c r="G7" s="77"/>
+      <c r="H7" s="77"/>
+      <c r="I7" s="54"/>
+      <c r="J7" s="55"/>
+      <c r="K7" s="56"/>
+      <c r="L7" s="57"/>
+      <c r="M7" s="58"/>
+      <c r="N7" s="58"/>
+      <c r="O7" s="58"/>
+      <c r="P7" s="58"/>
+      <c r="Q7" s="58"/>
+      <c r="R7" s="58"/>
+      <c r="S7" s="58"/>
+      <c r="T7" s="58"/>
+      <c r="U7" s="58"/>
+      <c r="V7" s="58"/>
+      <c r="W7" s="58"/>
+      <c r="X7" s="58"/>
+      <c r="Y7" s="58"/>
+      <c r="Z7" s="58"/>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="77"/>
+      <c r="A8" s="78"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
-      <c r="D8" s="78"/>
-      <c r="E8" s="71"/>
-      <c r="F8" s="71"/>
-      <c r="G8" s="71"/>
-      <c r="H8" s="71"/>
-      <c r="I8" s="71"/>
-      <c r="J8" s="79"/>
-      <c r="K8" s="79"/>
-      <c r="L8" s="56"/>
-      <c r="M8" s="57"/>
-      <c r="N8" s="57"/>
-      <c r="O8" s="57"/>
-      <c r="P8" s="57"/>
-      <c r="Q8" s="57"/>
-      <c r="R8" s="57"/>
-      <c r="S8" s="57"/>
-      <c r="T8" s="57"/>
-      <c r="U8" s="57"/>
-      <c r="V8" s="57"/>
-      <c r="W8" s="57"/>
-      <c r="X8" s="57"/>
-      <c r="Y8" s="57"/>
-      <c r="Z8" s="57"/>
+      <c r="D8" s="79"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="72"/>
+      <c r="H8" s="72"/>
+      <c r="I8" s="72"/>
+      <c r="J8" s="80"/>
+      <c r="K8" s="80"/>
+      <c r="L8" s="57"/>
+      <c r="M8" s="58"/>
+      <c r="N8" s="58"/>
+      <c r="O8" s="58"/>
+      <c r="P8" s="58"/>
+      <c r="Q8" s="58"/>
+      <c r="R8" s="58"/>
+      <c r="S8" s="58"/>
+      <c r="T8" s="58"/>
+      <c r="U8" s="58"/>
+      <c r="V8" s="58"/>
+      <c r="W8" s="58"/>
+      <c r="X8" s="58"/>
+      <c r="Y8" s="58"/>
+      <c r="Z8" s="58"/>
     </row>
     <row r="9" ht="12.0" customHeight="1">
-      <c r="A9" s="80" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="81" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="80" t="s">
+      <c r="A9" s="81" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="82" t="s">
+      <c r="B9" s="82" t="s">
         <v>32</v>
+      </c>
+      <c r="C9" s="81" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="83" t="s">
+        <v>34</v>
       </c>
       <c r="E9" s="42"/>
       <c r="F9" s="42"/>
-      <c r="G9" s="83"/>
-      <c r="H9" s="80" t="s">
-        <v>33</v>
-      </c>
-      <c r="I9" s="84" t="s">
-        <v>34</v>
-      </c>
-      <c r="J9" s="84" t="s">
+      <c r="G9" s="84"/>
+      <c r="H9" s="81" t="s">
         <v>35</v>
       </c>
-      <c r="K9" s="84" t="s">
+      <c r="I9" s="85" t="s">
         <v>36</v>
       </c>
-      <c r="L9" s="85"/>
-      <c r="M9" s="86"/>
-      <c r="N9" s="86"/>
-      <c r="O9" s="86"/>
-      <c r="P9" s="86"/>
-      <c r="Q9" s="86"/>
-      <c r="R9" s="86"/>
-      <c r="S9" s="86"/>
-      <c r="T9" s="86"/>
-      <c r="U9" s="86"/>
-      <c r="V9" s="86"/>
-      <c r="W9" s="86"/>
-      <c r="X9" s="86"/>
-      <c r="Y9" s="86"/>
-      <c r="Z9" s="86"/>
+      <c r="J9" s="85" t="s">
+        <v>37</v>
+      </c>
+      <c r="K9" s="85" t="s">
+        <v>38</v>
+      </c>
+      <c r="L9" s="86"/>
+      <c r="M9" s="87"/>
+      <c r="N9" s="87"/>
+      <c r="O9" s="87"/>
+      <c r="P9" s="87"/>
+      <c r="Q9" s="87"/>
+      <c r="R9" s="87"/>
+      <c r="S9" s="87"/>
+      <c r="T9" s="87"/>
+      <c r="U9" s="87"/>
+      <c r="V9" s="87"/>
+      <c r="W9" s="87"/>
+      <c r="X9" s="87"/>
+      <c r="Y9" s="87"/>
+      <c r="Z9" s="87"/>
     </row>
     <row r="10" ht="12.0" customHeight="1">
-      <c r="A10" s="87"/>
-      <c r="B10" s="87"/>
-      <c r="C10" s="87"/>
-      <c r="D10" s="88"/>
-      <c r="E10" s="89"/>
-      <c r="F10" s="89"/>
-      <c r="G10" s="90"/>
-      <c r="H10" s="87"/>
-      <c r="I10" s="87"/>
-      <c r="J10" s="87"/>
-      <c r="K10" s="87"/>
-      <c r="L10" s="56"/>
-      <c r="M10" s="57"/>
-      <c r="N10" s="57"/>
-      <c r="O10" s="57"/>
-      <c r="P10" s="57"/>
-      <c r="Q10" s="57"/>
-      <c r="R10" s="57"/>
-      <c r="S10" s="57"/>
-      <c r="T10" s="57"/>
-      <c r="U10" s="57"/>
-      <c r="V10" s="57"/>
-      <c r="W10" s="57"/>
-      <c r="X10" s="57"/>
-      <c r="Y10" s="57"/>
-      <c r="Z10" s="57"/>
+      <c r="A10" s="88"/>
+      <c r="B10" s="88"/>
+      <c r="C10" s="88"/>
+      <c r="D10" s="89"/>
+      <c r="E10" s="90"/>
+      <c r="F10" s="90"/>
+      <c r="G10" s="91"/>
+      <c r="H10" s="88"/>
+      <c r="I10" s="88"/>
+      <c r="J10" s="88"/>
+      <c r="K10" s="88"/>
+      <c r="L10" s="57"/>
+      <c r="M10" s="58"/>
+      <c r="N10" s="58"/>
+      <c r="O10" s="58"/>
+      <c r="P10" s="58"/>
+      <c r="Q10" s="58"/>
+      <c r="R10" s="58"/>
+      <c r="S10" s="58"/>
+      <c r="T10" s="58"/>
+      <c r="U10" s="58"/>
+      <c r="V10" s="58"/>
+      <c r="W10" s="58"/>
+      <c r="X10" s="58"/>
+      <c r="Y10" s="58"/>
+      <c r="Z10" s="58"/>
     </row>
     <row r="11" ht="13.5" customHeight="1">
-      <c r="A11" s="91"/>
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="60"/>
-      <c r="G11" s="60"/>
-      <c r="H11" s="60"/>
-      <c r="I11" s="60"/>
-      <c r="J11" s="60"/>
-      <c r="K11" s="92"/>
-      <c r="L11" s="93"/>
-      <c r="M11" s="93"/>
-      <c r="N11" s="93"/>
-      <c r="O11" s="93"/>
-      <c r="P11" s="93"/>
-      <c r="Q11" s="93"/>
-      <c r="R11" s="93"/>
-      <c r="S11" s="93"/>
-      <c r="T11" s="93"/>
-      <c r="U11" s="93"/>
-      <c r="V11" s="93"/>
-      <c r="W11" s="93"/>
-      <c r="X11" s="93"/>
-      <c r="Y11" s="93"/>
-      <c r="Z11" s="93"/>
+      <c r="A11" s="92"/>
+      <c r="B11" s="61"/>
+      <c r="C11" s="61"/>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
+      <c r="I11" s="61"/>
+      <c r="J11" s="61"/>
+      <c r="K11" s="93"/>
+      <c r="L11" s="94"/>
+      <c r="M11" s="94"/>
+      <c r="N11" s="94"/>
+      <c r="O11" s="94"/>
+      <c r="P11" s="94"/>
+      <c r="Q11" s="94"/>
+      <c r="R11" s="94"/>
+      <c r="S11" s="94"/>
+      <c r="T11" s="94"/>
+      <c r="U11" s="94"/>
+      <c r="V11" s="94"/>
+      <c r="W11" s="94"/>
+      <c r="X11" s="94"/>
+      <c r="Y11" s="94"/>
+      <c r="Z11" s="94"/>
     </row>
     <row r="12" ht="13.5" customHeight="1">
-      <c r="A12" s="94"/>
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="60"/>
-      <c r="I12" s="60"/>
-      <c r="J12" s="60"/>
-      <c r="K12" s="92"/>
-      <c r="L12" s="95"/>
-      <c r="M12" s="95"/>
-      <c r="N12" s="95"/>
-      <c r="O12" s="95"/>
-      <c r="P12" s="95"/>
-      <c r="Q12" s="95"/>
-      <c r="R12" s="95"/>
-      <c r="S12" s="95"/>
-      <c r="T12" s="95"/>
-      <c r="U12" s="95"/>
-      <c r="V12" s="95"/>
-      <c r="W12" s="95"/>
-      <c r="X12" s="95"/>
-      <c r="Y12" s="95"/>
-      <c r="Z12" s="95"/>
+      <c r="A12" s="112"/>
+      <c r="B12" s="61"/>
+      <c r="C12" s="61"/>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="61"/>
+      <c r="G12" s="61"/>
+      <c r="H12" s="61"/>
+      <c r="I12" s="61"/>
+      <c r="J12" s="61"/>
+      <c r="K12" s="93"/>
+      <c r="L12" s="96"/>
+      <c r="M12" s="96"/>
+      <c r="N12" s="96"/>
+      <c r="O12" s="96"/>
+      <c r="P12" s="96"/>
+      <c r="Q12" s="96"/>
+      <c r="R12" s="96"/>
+      <c r="S12" s="96"/>
+      <c r="T12" s="96"/>
+      <c r="U12" s="96"/>
+      <c r="V12" s="96"/>
+      <c r="W12" s="96"/>
+      <c r="X12" s="96"/>
+      <c r="Y12" s="96"/>
+      <c r="Z12" s="96"/>
     </row>
     <row r="13" ht="13.5" customHeight="1" outlineLevel="1">
-      <c r="A13" s="96"/>
-      <c r="B13" s="97"/>
-      <c r="C13" s="98"/>
-      <c r="D13" s="99"/>
-      <c r="E13" s="60"/>
-      <c r="F13" s="60"/>
-      <c r="G13" s="100"/>
-      <c r="H13" s="101"/>
-      <c r="I13" s="102"/>
-      <c r="J13" s="98" t="s">
-        <v>25</v>
+      <c r="A13" s="113"/>
+      <c r="B13" s="114"/>
+      <c r="C13" s="104"/>
+      <c r="D13" s="107"/>
+      <c r="E13" s="61"/>
+      <c r="F13" s="61"/>
+      <c r="G13" s="101"/>
+      <c r="H13" s="108"/>
+      <c r="I13" s="103"/>
+      <c r="J13" s="104" t="s">
+        <v>27</v>
       </c>
-      <c r="K13" s="98"/>
-      <c r="L13" s="95"/>
-      <c r="M13" s="95"/>
-      <c r="N13" s="95"/>
-      <c r="O13" s="95"/>
-      <c r="P13" s="95"/>
-      <c r="Q13" s="95"/>
-      <c r="R13" s="95"/>
-      <c r="S13" s="95"/>
-      <c r="T13" s="95"/>
-      <c r="U13" s="95"/>
-      <c r="V13" s="95"/>
-      <c r="W13" s="95"/>
-      <c r="X13" s="95"/>
-      <c r="Y13" s="95"/>
-      <c r="Z13" s="95"/>
+      <c r="K13" s="104"/>
+      <c r="L13" s="96"/>
+      <c r="M13" s="96"/>
+      <c r="N13" s="96"/>
+      <c r="O13" s="96"/>
+      <c r="P13" s="96"/>
+      <c r="Q13" s="96"/>
+      <c r="R13" s="96"/>
+      <c r="S13" s="96"/>
+      <c r="T13" s="96"/>
+      <c r="U13" s="96"/>
+      <c r="V13" s="96"/>
+      <c r="W13" s="96"/>
+      <c r="X13" s="96"/>
+      <c r="Y13" s="96"/>
+      <c r="Z13" s="96"/>
     </row>
     <row r="14" ht="13.5" customHeight="1" outlineLevel="1">
-      <c r="A14" s="103"/>
-      <c r="B14" s="60"/>
-      <c r="C14" s="104"/>
-      <c r="D14" s="105"/>
-      <c r="E14" s="105"/>
-      <c r="F14" s="105"/>
-      <c r="G14" s="105"/>
-      <c r="H14" s="105"/>
-      <c r="I14" s="105"/>
-      <c r="J14" s="105"/>
-      <c r="K14" s="106"/>
-      <c r="L14" s="95"/>
-      <c r="M14" s="95"/>
-      <c r="N14" s="95"/>
-      <c r="O14" s="95"/>
-      <c r="P14" s="95"/>
-      <c r="Q14" s="95"/>
-      <c r="R14" s="95"/>
-      <c r="S14" s="95"/>
-      <c r="T14" s="95"/>
-      <c r="U14" s="95"/>
-      <c r="V14" s="95"/>
-      <c r="W14" s="95"/>
-      <c r="X14" s="95"/>
-      <c r="Y14" s="95"/>
-      <c r="Z14" s="95"/>
+      <c r="A14" s="115"/>
+      <c r="B14" s="61"/>
+      <c r="C14" s="116"/>
+      <c r="D14" s="117"/>
+      <c r="E14" s="117"/>
+      <c r="F14" s="117"/>
+      <c r="G14" s="117"/>
+      <c r="H14" s="117"/>
+      <c r="I14" s="117"/>
+      <c r="J14" s="117"/>
+      <c r="K14" s="118"/>
+      <c r="L14" s="96"/>
+      <c r="M14" s="96"/>
+      <c r="N14" s="96"/>
+      <c r="O14" s="96"/>
+      <c r="P14" s="96"/>
+      <c r="Q14" s="96"/>
+      <c r="R14" s="96"/>
+      <c r="S14" s="96"/>
+      <c r="T14" s="96"/>
+      <c r="U14" s="96"/>
+      <c r="V14" s="96"/>
+      <c r="W14" s="96"/>
+      <c r="X14" s="96"/>
+      <c r="Y14" s="96"/>
+      <c r="Z14" s="96"/>
     </row>
     <row r="15" ht="63.75" customHeight="1" outlineLevel="1">
-      <c r="A15" s="96"/>
-      <c r="B15" s="107"/>
-      <c r="C15" s="108"/>
-      <c r="D15" s="109"/>
-      <c r="E15" s="60"/>
-      <c r="F15" s="60"/>
-      <c r="G15" s="100"/>
-      <c r="H15" s="101"/>
-      <c r="I15" s="99"/>
-      <c r="J15" s="98" t="s">
-        <v>25</v>
+      <c r="A15" s="113"/>
+      <c r="B15" s="119"/>
+      <c r="C15" s="120"/>
+      <c r="D15" s="121"/>
+      <c r="E15" s="61"/>
+      <c r="F15" s="61"/>
+      <c r="G15" s="101"/>
+      <c r="H15" s="108"/>
+      <c r="I15" s="107"/>
+      <c r="J15" s="104" t="s">
+        <v>27</v>
       </c>
-      <c r="K15" s="98"/>
-      <c r="L15" s="95"/>
-      <c r="M15" s="95"/>
-      <c r="N15" s="95"/>
-      <c r="O15" s="95"/>
-      <c r="P15" s="95"/>
-      <c r="Q15" s="95"/>
-      <c r="R15" s="95"/>
-      <c r="S15" s="95"/>
-      <c r="T15" s="95"/>
-      <c r="U15" s="95"/>
-      <c r="V15" s="95"/>
-      <c r="W15" s="95"/>
-      <c r="X15" s="95"/>
-      <c r="Y15" s="95"/>
-      <c r="Z15" s="95"/>
+      <c r="K15" s="104"/>
+      <c r="L15" s="96"/>
+      <c r="M15" s="96"/>
+      <c r="N15" s="96"/>
+      <c r="O15" s="96"/>
+      <c r="P15" s="96"/>
+      <c r="Q15" s="96"/>
+      <c r="R15" s="96"/>
+      <c r="S15" s="96"/>
+      <c r="T15" s="96"/>
+      <c r="U15" s="96"/>
+      <c r="V15" s="96"/>
+      <c r="W15" s="96"/>
+      <c r="X15" s="96"/>
+      <c r="Y15" s="96"/>
+      <c r="Z15" s="96"/>
     </row>
     <row r="16" ht="13.5" customHeight="1" outlineLevel="1">
-      <c r="A16" s="103"/>
-      <c r="B16" s="60"/>
-      <c r="C16" s="104"/>
-      <c r="D16" s="105"/>
-      <c r="E16" s="105"/>
-      <c r="F16" s="105"/>
-      <c r="G16" s="105"/>
-      <c r="H16" s="105"/>
-      <c r="I16" s="105"/>
-      <c r="J16" s="105"/>
-      <c r="K16" s="106"/>
-      <c r="L16" s="95"/>
-      <c r="M16" s="95"/>
-      <c r="N16" s="95"/>
-      <c r="O16" s="95"/>
-      <c r="P16" s="95"/>
-      <c r="Q16" s="95"/>
-      <c r="R16" s="95"/>
-      <c r="S16" s="95"/>
-      <c r="T16" s="95"/>
-      <c r="U16" s="95"/>
-      <c r="V16" s="95"/>
-      <c r="W16" s="95"/>
-      <c r="X16" s="95"/>
-      <c r="Y16" s="95"/>
-      <c r="Z16" s="95"/>
+      <c r="A16" s="115"/>
+      <c r="B16" s="61"/>
+      <c r="C16" s="116"/>
+      <c r="D16" s="117"/>
+      <c r="E16" s="117"/>
+      <c r="F16" s="117"/>
+      <c r="G16" s="117"/>
+      <c r="H16" s="117"/>
+      <c r="I16" s="117"/>
+      <c r="J16" s="117"/>
+      <c r="K16" s="118"/>
+      <c r="L16" s="96"/>
+      <c r="M16" s="96"/>
+      <c r="N16" s="96"/>
+      <c r="O16" s="96"/>
+      <c r="P16" s="96"/>
+      <c r="Q16" s="96"/>
+      <c r="R16" s="96"/>
+      <c r="S16" s="96"/>
+      <c r="T16" s="96"/>
+      <c r="U16" s="96"/>
+      <c r="V16" s="96"/>
+      <c r="W16" s="96"/>
+      <c r="X16" s="96"/>
+      <c r="Y16" s="96"/>
+      <c r="Z16" s="96"/>
     </row>
     <row r="17" ht="63.75" customHeight="1" outlineLevel="1">
-      <c r="A17" s="96"/>
-      <c r="B17" s="110"/>
-      <c r="C17" s="98"/>
-      <c r="D17" s="109"/>
-      <c r="E17" s="60"/>
-      <c r="F17" s="60"/>
-      <c r="G17" s="100"/>
-      <c r="H17" s="101"/>
-      <c r="I17" s="99"/>
-      <c r="J17" s="98" t="s">
-        <v>25</v>
+      <c r="A17" s="113"/>
+      <c r="B17" s="122"/>
+      <c r="C17" s="104"/>
+      <c r="D17" s="121"/>
+      <c r="E17" s="61"/>
+      <c r="F17" s="61"/>
+      <c r="G17" s="101"/>
+      <c r="H17" s="108"/>
+      <c r="I17" s="107"/>
+      <c r="J17" s="104" t="s">
+        <v>27</v>
       </c>
-      <c r="K17" s="98"/>
-      <c r="L17" s="95"/>
-      <c r="M17" s="95"/>
-      <c r="N17" s="95"/>
-      <c r="O17" s="95"/>
-      <c r="P17" s="95"/>
-      <c r="Q17" s="95"/>
-      <c r="R17" s="95"/>
-      <c r="S17" s="95"/>
-      <c r="T17" s="95"/>
-      <c r="U17" s="95"/>
-      <c r="V17" s="95"/>
-      <c r="W17" s="95"/>
-      <c r="X17" s="95"/>
-      <c r="Y17" s="95"/>
-      <c r="Z17" s="95"/>
+      <c r="K17" s="104"/>
+      <c r="L17" s="96"/>
+      <c r="M17" s="96"/>
+      <c r="N17" s="96"/>
+      <c r="O17" s="96"/>
+      <c r="P17" s="96"/>
+      <c r="Q17" s="96"/>
+      <c r="R17" s="96"/>
+      <c r="S17" s="96"/>
+      <c r="T17" s="96"/>
+      <c r="U17" s="96"/>
+      <c r="V17" s="96"/>
+      <c r="W17" s="96"/>
+      <c r="X17" s="96"/>
+      <c r="Y17" s="96"/>
+      <c r="Z17" s="96"/>
     </row>
     <row r="18" ht="12.0" customHeight="1">
       <c r="J18" s="11"/>
@@ -43787,40 +44060,40 @@
   </cols>
   <sheetData>
     <row r="1" ht="12.75" customHeight="1">
-      <c r="A1" s="111" t="s">
-        <v>43</v>
+      <c r="A1" s="123" t="s">
+        <v>66</v>
       </c>
-      <c r="B1" s="112"/>
+      <c r="B1" s="124"/>
       <c r="C1" s="11"/>
       <c r="D1" s="11"/>
       <c r="E1" s="11"/>
       <c r="F1" s="11"/>
-      <c r="G1" s="113"/>
+      <c r="G1" s="125"/>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" s="111"/>
-      <c r="B2" s="112"/>
+      <c r="A2" s="123"/>
+      <c r="B2" s="124"/>
       <c r="C2" s="11"/>
       <c r="D2" s="11"/>
       <c r="E2" s="11"/>
       <c r="F2" s="11"/>
-      <c r="G2" s="113"/>
+      <c r="G2" s="125"/>
     </row>
     <row r="3" ht="12.75" customHeight="1">
       <c r="B3" s="11" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="11"/>
       <c r="E3" s="11"/>
       <c r="F3" s="11"/>
-      <c r="G3" s="113"/>
+      <c r="G3" s="125"/>
     </row>
     <row r="4" ht="12.75" customHeight="1">
       <c r="B4" s="11" t="s">
-        <v>45</v>
+        <v>68</v>
       </c>
-      <c r="C4" s="114"/>
+      <c r="C4" s="126"/>
       <c r="D4" s="11"/>
       <c r="E4" s="11"/>
       <c r="F4" s="11"/>
@@ -43846,142 +44119,142 @@
     </row>
     <row r="7" ht="12.75" customHeight="1">
       <c r="A7" s="11"/>
-      <c r="B7" s="115" t="s">
-        <v>46</v>
+      <c r="B7" s="127" t="s">
+        <v>69</v>
       </c>
-      <c r="C7" s="116" t="s">
-        <v>47</v>
+      <c r="C7" s="128" t="s">
+        <v>70</v>
       </c>
-      <c r="D7" s="117" t="s">
-        <v>25</v>
-      </c>
-      <c r="E7" s="116" t="s">
+      <c r="D7" s="129" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="116" t="s">
-        <v>26</v>
+      <c r="E7" s="128" t="s">
+        <v>29</v>
       </c>
-      <c r="G7" s="118" t="s">
-        <v>48</v>
+      <c r="F7" s="128" t="s">
+        <v>28</v>
       </c>
+      <c r="G7" s="130" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="8" ht="12.75" customHeight="1">
-      <c r="A8" s="119"/>
-      <c r="B8" s="120">
+      <c r="A8" s="131"/>
+      <c r="B8" s="132">
         <v>1.0</v>
       </c>
-      <c r="C8" s="121" t="str">
-        <f>Borrow!B4</f>
+      <c r="C8" s="133" t="str">
+        <f>'Mượn sách'!B4</f>
         <v>CR100 - Export to excel</v>
       </c>
-      <c r="D8" s="122">
-        <f>Borrow!B6 + Return!B6 + Search!B6 + Database!B6</f>
+      <c r="D8" s="134">
+        <f>'Mượn sách'!B6 + 'Trả sách'!B6 + 'Tìm kiếm sách'!B6 + 'Cơ sở dữ liệu'!B6</f>
         <v>12</v>
       </c>
-      <c r="E8" s="121">
-        <f>Borrow!B7 +Return!B7+Search!B7</f>
+      <c r="E8" s="133">
+        <f>'Mượn sách'!B7 +'Trả sách'!B7+'Tìm kiếm sách'!B7</f>
         <v>0</v>
       </c>
-      <c r="F8" s="121">
-        <f>Borrow!D6</f>
+      <c r="F8" s="133">
+        <f>'Mượn sách'!D6</f>
         <v>0</v>
       </c>
-      <c r="G8" s="122">
-        <f>Borrow!D7+Return!D7 + Search!D7 + Database!D7</f>
-        <v>-60</v>
+      <c r="G8" s="134">
+        <f>'Mượn sách'!D7+'Trả sách'!D7 + 'Tìm kiếm sách'!D7 + 'Cơ sở dữ liệu'!D7</f>
+        <v>-55</v>
       </c>
-      <c r="H8" s="123"/>
-      <c r="I8" s="123"/>
-      <c r="J8" s="123"/>
-      <c r="K8" s="123"/>
-      <c r="L8" s="123"/>
-      <c r="M8" s="123"/>
-      <c r="N8" s="123"/>
-      <c r="O8" s="123"/>
-      <c r="P8" s="123"/>
-      <c r="Q8" s="123"/>
-      <c r="R8" s="123"/>
-      <c r="S8" s="123"/>
-      <c r="T8" s="123"/>
-      <c r="U8" s="123"/>
-      <c r="V8" s="123"/>
-      <c r="W8" s="123"/>
-      <c r="X8" s="123"/>
-      <c r="Y8" s="123"/>
-      <c r="Z8" s="123"/>
+      <c r="H8" s="135"/>
+      <c r="I8" s="135"/>
+      <c r="J8" s="135"/>
+      <c r="K8" s="135"/>
+      <c r="L8" s="135"/>
+      <c r="M8" s="135"/>
+      <c r="N8" s="135"/>
+      <c r="O8" s="135"/>
+      <c r="P8" s="135"/>
+      <c r="Q8" s="135"/>
+      <c r="R8" s="135"/>
+      <c r="S8" s="135"/>
+      <c r="T8" s="135"/>
+      <c r="U8" s="135"/>
+      <c r="V8" s="135"/>
+      <c r="W8" s="135"/>
+      <c r="X8" s="135"/>
+      <c r="Y8" s="135"/>
+      <c r="Z8" s="135"/>
     </row>
     <row r="9" ht="12.75" customHeight="1">
       <c r="A9" s="11"/>
-      <c r="B9" s="124"/>
-      <c r="C9" s="125"/>
-      <c r="D9" s="126"/>
-      <c r="E9" s="127"/>
-      <c r="F9" s="127"/>
-      <c r="G9" s="128"/>
+      <c r="B9" s="136"/>
+      <c r="C9" s="137"/>
+      <c r="D9" s="138"/>
+      <c r="E9" s="139"/>
+      <c r="F9" s="139"/>
+      <c r="G9" s="140"/>
     </row>
     <row r="10" ht="12.75" customHeight="1">
       <c r="A10" s="11"/>
-      <c r="B10" s="129"/>
-      <c r="C10" s="130" t="s">
-        <v>49</v>
+      <c r="B10" s="141"/>
+      <c r="C10" s="142" t="s">
+        <v>72</v>
       </c>
-      <c r="D10" s="131">
+      <c r="D10" s="143">
         <f t="shared" ref="D10:G10" si="1">SUM(D6:D9)</f>
         <v>12</v>
       </c>
-      <c r="E10" s="131">
+      <c r="E10" s="143">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="F10" s="131">
+      <c r="F10" s="143">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="G10" s="132">
+      <c r="G10" s="144">
         <f t="shared" si="1"/>
-        <v>-60</v>
+        <v>-55</v>
       </c>
     </row>
     <row r="11" ht="12.75" customHeight="1">
       <c r="A11" s="11"/>
-      <c r="B11" s="133"/>
+      <c r="B11" s="145"/>
       <c r="C11" s="11"/>
-      <c r="D11" s="134"/>
-      <c r="E11" s="135"/>
-      <c r="F11" s="135"/>
-      <c r="G11" s="135"/>
+      <c r="D11" s="146"/>
+      <c r="E11" s="147"/>
+      <c r="F11" s="147"/>
+      <c r="G11" s="147"/>
     </row>
     <row r="12" ht="12.75" customHeight="1">
       <c r="A12" s="11"/>
       <c r="B12" s="11"/>
       <c r="C12" s="11" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="D12" s="11"/>
-      <c r="E12" s="136">
+      <c r="E12" s="148">
         <f>(D10+E10)*100/G10</f>
-        <v>-20</v>
+        <v>-21.81818182</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
-      <c r="G12" s="137"/>
+      <c r="G12" s="149"/>
     </row>
     <row r="13" ht="12.75" customHeight="1">
       <c r="A13" s="11"/>
       <c r="B13" s="11"/>
       <c r="C13" s="11" t="s">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="D13" s="11"/>
-      <c r="E13" s="136">
+      <c r="E13" s="148">
         <f>D10*100/G10</f>
-        <v>-20</v>
+        <v>-21.81818182</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>51</v>
+        <v>74</v>
       </c>
-      <c r="G13" s="137"/>
+      <c r="G13" s="149"/>
     </row>
     <row r="14" ht="12.75" customHeight="1"/>
     <row r="15" ht="12.75" customHeight="1"/>

</xml_diff>